<commit_message>
Inclui 26815 LABORATORIO DE ANALISE BIOMECANICA DO MOVIMENTO HUMANO
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
+++ b/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
@@ -341,7 +341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E429"/>
+  <dimension ref="A1:E430"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="52" customWidth="1" style="4" min="1" max="1"/>
@@ -3005,1520 +3005,1529 @@
       </c>
     </row>
     <row r="272" ht="15.75" customHeight="1" s="4">
-      <c r="B272" s="3" t="inlineStr">
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>LABORATORIO DE ANALISE BIOMECANICA DO MOVIMENTO HUMANO</t>
+        </is>
+      </c>
+      <c r="E272" t="n">
+        <v>26815</v>
+      </c>
+    </row>
+    <row r="273" ht="15.75" customHeight="1" s="4">
+      <c r="B273" s="3" t="inlineStr">
         <is>
           <t>COORDENACAO</t>
         </is>
-      </c>
-    </row>
-    <row r="273" ht="15.75" customHeight="1" s="4">
-      <c r="C273" s="3" t="inlineStr">
-        <is>
-          <t>SALA COORDENAÇÃO DE GRADUACAO EM EDUCACAO FISICA - SALA 1</t>
-        </is>
-      </c>
-      <c r="E273" s="3" t="n">
-        <v>26811</v>
       </c>
     </row>
     <row r="274" ht="15.75" customHeight="1" s="4">
       <c r="C274" s="3" t="inlineStr">
         <is>
-          <t>SALA COORDENAÇÃO DE GRADUACAO EM EDUCACAO FISICA - SALA 2</t>
+          <t>SALA COORDENAÇÃO DE GRADUACAO EM EDUCACAO FISICA - SALA 1</t>
         </is>
       </c>
       <c r="E274" s="3" t="n">
-        <v>26812</v>
+        <v>26811</v>
       </c>
     </row>
     <row r="275" ht="15.75" customHeight="1" s="4">
       <c r="C275" s="3" t="inlineStr">
         <is>
-          <t>SALA COORDENAÇÃO DE GRADUACAO EM EDUCACAO FISICA - SALA 3</t>
+          <t>SALA COORDENAÇÃO DE GRADUACAO EM EDUCACAO FISICA - SALA 2</t>
         </is>
       </c>
       <c r="E275" s="3" t="n">
-        <v>26813</v>
+        <v>26812</v>
       </c>
     </row>
     <row r="276" ht="15.75" customHeight="1" s="4">
       <c r="C276" s="3" t="inlineStr">
         <is>
+          <t>SALA COORDENAÇÃO DE GRADUACAO EM EDUCACAO FISICA - SALA 3</t>
+        </is>
+      </c>
+      <c r="E276" s="3" t="n">
+        <v>26813</v>
+      </c>
+    </row>
+    <row r="277" ht="15.75" customHeight="1" s="4">
+      <c r="C277" s="3" t="inlineStr">
+        <is>
           <t>SALA COORDENAÇÃO DE GRADUACAO EM EDUCACAO FISICA - SALA 4</t>
         </is>
       </c>
-      <c r="E276" s="3" t="n">
+      <c r="E277" s="3" t="n">
         <v>26814</v>
       </c>
     </row>
-    <row r="277" ht="15.75" customHeight="1" s="4">
-      <c r="B277" s="3" t="inlineStr">
+    <row r="278" ht="15.75" customHeight="1" s="4">
+      <c r="B278" s="3" t="inlineStr">
         <is>
           <t>SALA COORDENAÇÃO DE GRADUACAO EM EDUCACAO FISICA</t>
         </is>
       </c>
-      <c r="E277" s="3" t="n">
+      <c r="E278" s="3" t="n">
         <v>26802</v>
       </c>
     </row>
-    <row r="278" ht="15.75" customHeight="1" s="4">
-      <c r="A278" s="3" t="inlineStr">
+    <row r="279" ht="15.75" customHeight="1" s="4">
+      <c r="A279" s="3" t="inlineStr">
         <is>
           <t>NUCLEO DE DIREITO</t>
         </is>
-      </c>
-    </row>
-    <row r="279" ht="15.75" customHeight="1" s="4">
-      <c r="B279" s="3" t="inlineStr">
-        <is>
-          <t>NUCLEO DE DIREITO</t>
-        </is>
-      </c>
-      <c r="E279" s="3" t="n">
-        <v>26900</v>
       </c>
     </row>
     <row r="280" ht="15.75" customHeight="1" s="4">
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>NUCLEO DE DIREITO - SALA DE AULA 1 - PRATICA JURIDICA</t>
+          <t>NUCLEO DE DIREITO</t>
         </is>
       </c>
       <c r="E280" s="3" t="n">
-        <v>26901</v>
+        <v>26900</v>
       </c>
     </row>
     <row r="281" ht="15.75" customHeight="1" s="4">
       <c r="B281" s="3" t="inlineStr">
         <is>
+          <t>NUCLEO DE DIREITO - SALA DE AULA 1 - PRATICA JURIDICA</t>
+        </is>
+      </c>
+      <c r="E281" s="3" t="n">
+        <v>26901</v>
+      </c>
+    </row>
+    <row r="282" ht="15.75" customHeight="1" s="4">
+      <c r="B282" s="3" t="inlineStr">
+        <is>
           <t>PAPRE - POSTO DE ATENDIMENTO PRÉ PROCESSUAL</t>
         </is>
       </c>
-      <c r="E281" s="3" t="n">
+      <c r="E282" s="3" t="n">
         <v>26902</v>
       </c>
     </row>
-    <row r="282" ht="15.75" customHeight="1" s="4">
-      <c r="A282" s="3" t="inlineStr">
+    <row r="283" ht="15.75" customHeight="1" s="4">
+      <c r="A283" s="3" t="inlineStr">
         <is>
           <t>DIRETORIA DE ADMINISTRACAO E PLANEJAMENTO</t>
         </is>
-      </c>
-    </row>
-    <row r="283" ht="15.75" customHeight="1" s="4">
-      <c r="B283" s="3" t="inlineStr">
-        <is>
-          <t>DIRETORIA DE ADMINISTRACAO E PLANEJAMENTO</t>
-        </is>
-      </c>
-      <c r="E283" s="3" t="n">
-        <v>30000</v>
       </c>
     </row>
     <row r="284" ht="15.75" customHeight="1" s="4">
       <c r="B284" s="3" t="inlineStr">
         <is>
+          <t>DIRETORIA DE ADMINISTRACAO E PLANEJAMENTO</t>
+        </is>
+      </c>
+      <c r="E284" s="3" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="285" ht="15.75" customHeight="1" s="4">
+      <c r="B285" s="3" t="inlineStr">
+        <is>
           <t>PREDIO ADMINISTRATIVO</t>
         </is>
-      </c>
-    </row>
-    <row r="285" ht="15.75" customHeight="1" s="4">
-      <c r="C285" s="3" t="inlineStr">
-        <is>
-          <t>PRÉDIO ADMINISTRATIVO - SALA DE REUNIAO</t>
-        </is>
-      </c>
-      <c r="E285" s="3" t="n">
-        <v>30001</v>
       </c>
     </row>
     <row r="286" ht="15.75" customHeight="1" s="4">
       <c r="C286" s="3" t="inlineStr">
         <is>
-          <t>PREDIO ADMINISTRATIVO - SALA DIRETORIA DE ADMINISTRACAO</t>
+          <t>PRÉDIO ADMINISTRATIVO - SALA DE REUNIAO</t>
         </is>
       </c>
       <c r="E286" s="3" t="n">
-        <v>30002</v>
+        <v>30001</v>
       </c>
     </row>
     <row r="287" ht="15.75" customHeight="1" s="4">
       <c r="C287" s="3" t="inlineStr">
         <is>
-          <t>PREDIO ADMINISTRATIVO - CASU</t>
+          <t>PREDIO ADMINISTRATIVO - SALA DIRETORIA DE ADMINISTRACAO</t>
         </is>
       </c>
       <c r="E287" s="3" t="n">
-        <v>30003</v>
+        <v>30002</v>
       </c>
     </row>
     <row r="288" ht="15.75" customHeight="1" s="4">
       <c r="C288" s="3" t="inlineStr">
         <is>
-          <t>PRÉDIO ADMINISTRATIVO - COPA</t>
+          <t>PREDIO ADMINISTRATIVO - CASU</t>
         </is>
       </c>
       <c r="E288" s="3" t="n">
-        <v>30004</v>
+        <v>30003</v>
       </c>
     </row>
     <row r="289" ht="15.75" customHeight="1" s="4">
       <c r="C289" s="3" t="inlineStr">
         <is>
-          <t>PRÉDIO ADMINISTRATIVO - COPA - DEPÓSITO (INSTRUMENTOS MUSICAIS)</t>
+          <t>PRÉDIO ADMINISTRATIVO - COPA</t>
         </is>
       </c>
       <c r="E289" s="3" t="n">
-        <v>30005</v>
+        <v>30004</v>
       </c>
     </row>
     <row r="290" ht="15.75" customHeight="1" s="4">
       <c r="C290" s="3" t="inlineStr">
         <is>
-          <t>PRÉDIO ADMINISTRATIVO - COPA - SALA DML TERCEIRIZADOS</t>
+          <t>PRÉDIO ADMINISTRATIVO - COPA - DEPÓSITO (INSTRUMENTOS MUSICAIS)</t>
         </is>
       </c>
       <c r="E290" s="3" t="n">
-        <v>30006</v>
+        <v>30005</v>
       </c>
     </row>
     <row r="291" ht="15.75" customHeight="1" s="4">
       <c r="C291" s="3" t="inlineStr">
         <is>
+          <t>PRÉDIO ADMINISTRATIVO - COPA - SALA DML TERCEIRIZADOS</t>
+        </is>
+      </c>
+      <c r="E291" s="3" t="n">
+        <v>30006</v>
+      </c>
+    </row>
+    <row r="292" ht="15.75" customHeight="1" s="4">
+      <c r="C292" s="3" t="inlineStr">
+        <is>
           <t>PRÉDIO ADMINISTRATIVO - SALA TELEFONISTA</t>
         </is>
       </c>
-      <c r="E291" s="3" t="n">
+      <c r="E292" s="3" t="n">
         <v>30007</v>
-      </c>
-    </row>
-    <row r="292" ht="15.75" customHeight="1" s="4">
-      <c r="B292" s="3" t="inlineStr">
-        <is>
-          <t>GUARITA 1 - IGREJINHA</t>
-        </is>
-      </c>
-      <c r="E292" s="3" t="n">
-        <v>30008</v>
       </c>
     </row>
     <row r="293" ht="15.75" customHeight="1" s="4">
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>GUARITA 2 - AGRICULTURA</t>
+          <t>GUARITA 1 - IGREJINHA</t>
         </is>
       </c>
       <c r="E293" s="3" t="n">
-        <v>30009</v>
+        <v>30008</v>
       </c>
     </row>
     <row r="294" ht="15.75" customHeight="1" s="4">
       <c r="B294" s="3" t="inlineStr">
         <is>
+          <t>GUARITA 2 - AGRICULTURA</t>
+        </is>
+      </c>
+      <c r="E294" s="3" t="n">
+        <v>30009</v>
+      </c>
+    </row>
+    <row r="295" ht="15.75" customHeight="1" s="4">
+      <c r="B295" s="3" t="inlineStr">
+        <is>
           <t>POSTO DE VIGILANCIA / VIGILANTE</t>
         </is>
       </c>
-      <c r="E294" s="3" t="n">
+      <c r="E295" s="3" t="n">
         <v>30010</v>
       </c>
     </row>
-    <row r="295" ht="15.75" customHeight="1" s="4">
-      <c r="B295" s="0" t="inlineStr">
+    <row r="296" ht="15.75" customHeight="1" s="4">
+      <c r="B296" s="0" t="inlineStr">
         <is>
           <t>COORDENACAO GERAL DE ADMINISTRACAO E FINANCAS</t>
         </is>
       </c>
-      <c r="E295" s="0" t="n">
+      <c r="E296" s="0" t="n">
         <v>31000</v>
       </c>
     </row>
-    <row r="296" ht="15.75" customHeight="1" s="4">
-      <c r="B296" s="3" t="inlineStr">
+    <row r="297" ht="15.75" customHeight="1" s="4">
+      <c r="B297" s="3" t="inlineStr">
         <is>
           <t>ALMOXARIFADO</t>
         </is>
-      </c>
-    </row>
-    <row r="297" ht="15.75" customHeight="1" s="4">
-      <c r="C297" s="3" t="inlineStr">
-        <is>
-          <t>ALMOXARIFADO</t>
-        </is>
-      </c>
-      <c r="E297" s="3" t="n">
-        <v>31100</v>
       </c>
     </row>
     <row r="298" ht="15.75" customHeight="1" s="4">
       <c r="C298" s="3" t="inlineStr">
         <is>
+          <t>ALMOXARIFADO</t>
+        </is>
+      </c>
+      <c r="E298" s="3" t="n">
+        <v>31100</v>
+      </c>
+    </row>
+    <row r="299" ht="15.75" customHeight="1" s="4">
+      <c r="C299" s="3" t="inlineStr">
+        <is>
           <t>ALMOXARIFADO - SOTAO</t>
         </is>
       </c>
-      <c r="E298" s="3" t="n">
+      <c r="E299" s="3" t="n">
         <v>31101</v>
       </c>
     </row>
-    <row r="299" ht="15.75" customHeight="1" s="4">
-      <c r="B299" s="3" t="inlineStr">
+    <row r="300" ht="15.75" customHeight="1" s="4">
+      <c r="B300" s="3" t="inlineStr">
         <is>
           <t>PATRIMONIO</t>
         </is>
-      </c>
-    </row>
-    <row r="300" ht="15.75" customHeight="1" s="4">
-      <c r="C300" s="3" t="inlineStr">
-        <is>
-          <t>PATRIMONIO</t>
-        </is>
-      </c>
-      <c r="E300" s="3" t="n">
-        <v>31200</v>
       </c>
     </row>
     <row r="301" ht="15.75" customHeight="1" s="4">
       <c r="C301" s="3" t="inlineStr">
         <is>
-          <t>SALA PATRIMÔNIO</t>
+          <t>PATRIMONIO</t>
         </is>
       </c>
       <c r="E301" s="3" t="n">
-        <v>31201</v>
+        <v>31200</v>
       </c>
     </row>
     <row r="302" ht="15.75" customHeight="1" s="4">
       <c r="C302" s="3" t="inlineStr">
         <is>
-          <t>PATRIMONIO - GALPAO 1</t>
+          <t>SALA PATRIMÔNIO</t>
         </is>
       </c>
       <c r="E302" s="3" t="n">
-        <v>31202</v>
+        <v>31201</v>
       </c>
     </row>
     <row r="303" ht="15.75" customHeight="1" s="4">
       <c r="C303" s="3" t="inlineStr">
         <is>
-          <t>PATRIMONIO - GALPAO 2 - AVALIACAO</t>
+          <t>PATRIMONIO - GALPAO 1</t>
         </is>
       </c>
       <c r="E303" s="3" t="n">
-        <v>31203</v>
+        <v>31202</v>
       </c>
     </row>
     <row r="304" ht="15.75" customHeight="1" s="4">
       <c r="C304" s="3" t="inlineStr">
         <is>
-          <t>PATRIMONIO - GALPAO 2 - DOACAO</t>
+          <t>PATRIMONIO - GALPAO 2 - AVALIACAO</t>
         </is>
       </c>
       <c r="E304" s="3" t="n">
-        <v>31204</v>
+        <v>31203</v>
       </c>
     </row>
     <row r="305" ht="15.75" customHeight="1" s="4">
       <c r="C305" s="3" t="inlineStr">
         <is>
-          <t>GALPAO 2 - IRRECUPERAVEL/ANTIECONOMICO</t>
+          <t>PATRIMONIO - GALPAO 2 - DOACAO</t>
         </is>
       </c>
       <c r="E305" s="3" t="n">
-        <v>31205</v>
+        <v>31204</v>
       </c>
     </row>
     <row r="306" ht="15.75" customHeight="1" s="4">
       <c r="C306" s="3" t="inlineStr">
         <is>
-          <t>PATRIMONIO - LAVANDERIA - AVALIACAO</t>
+          <t>GALPAO 2 - IRRECUPERAVEL/ANTIECONOMICO</t>
         </is>
       </c>
       <c r="E306" s="3" t="n">
-        <v>31206</v>
+        <v>31205</v>
       </c>
     </row>
     <row r="307" ht="15.75" customHeight="1" s="4">
       <c r="C307" s="3" t="inlineStr">
         <is>
-          <t>PATRIMONIO - LAVANDERIA - DOACAO</t>
+          <t>PATRIMONIO - LAVANDERIA - AVALIACAO</t>
         </is>
       </c>
       <c r="E307" s="3" t="n">
-        <v>31207</v>
+        <v>31206</v>
       </c>
     </row>
     <row r="308" ht="15.75" customHeight="1" s="4">
       <c r="C308" s="3" t="inlineStr">
         <is>
-          <t>PATRIMONIO - LAVANDERIA - IRRECUPERÁVEL</t>
+          <t>PATRIMONIO - LAVANDERIA - DOACAO</t>
         </is>
       </c>
       <c r="E308" s="3" t="n">
-        <v>31208</v>
+        <v>31207</v>
       </c>
     </row>
     <row r="309" ht="15.75" customHeight="1" s="4">
       <c r="C309" s="3" t="inlineStr">
         <is>
-          <t>PATRIMONIO - ESCOLINHA</t>
+          <t>PATRIMONIO - LAVANDERIA - IRRECUPERÁVEL</t>
         </is>
       </c>
       <c r="E309" s="3" t="n">
-        <v>31209</v>
+        <v>31208</v>
       </c>
     </row>
     <row r="310" ht="15.75" customHeight="1" s="4">
       <c r="C310" s="3" t="inlineStr">
         <is>
-          <t>REAVALIACAO - MATERIAL DE CONSUMO</t>
+          <t>PATRIMONIO - ESCOLINHA</t>
         </is>
       </c>
       <c r="E310" s="3" t="n">
-        <v>31210</v>
+        <v>31209</v>
       </c>
     </row>
     <row r="311" ht="15.75" customHeight="1" s="4">
       <c r="C311" s="3" t="inlineStr">
         <is>
+          <t>REAVALIACAO - MATERIAL DE CONSUMO</t>
+        </is>
+      </c>
+      <c r="E311" s="3" t="n">
+        <v>31210</v>
+      </c>
+    </row>
+    <row r="312" ht="15.75" customHeight="1" s="4">
+      <c r="C312" s="3" t="inlineStr">
+        <is>
           <t>PATRIMONIO - GALPAO 2</t>
         </is>
       </c>
-      <c r="E311" s="3" t="n">
+      <c r="E312" s="3" t="n">
         <v>31211</v>
-      </c>
-    </row>
-    <row r="312" ht="15.75" customHeight="1" s="4">
-      <c r="C312" s="0" t="inlineStr">
-        <is>
-          <t>PATRIMONIO - GALPAO 3 - IRRECUPERAVEL/ANTIECONOMIC</t>
-        </is>
-      </c>
-      <c r="E312" s="0" t="n">
-        <v>31212</v>
       </c>
     </row>
     <row r="313" ht="15.75" customHeight="1" s="4">
       <c r="C313" s="0" t="inlineStr">
         <is>
+          <t>PATRIMONIO - GALPAO 3 - IRRECUPERAVEL/ANTIECONOMIC</t>
+        </is>
+      </c>
+      <c r="E313" s="0" t="n">
+        <v>31212</v>
+      </c>
+    </row>
+    <row r="314" ht="15.75" customHeight="1" s="4">
+      <c r="C314" s="0" t="inlineStr">
+        <is>
           <t>PATRIMONIO - GALPAO 3</t>
         </is>
       </c>
-      <c r="E313" s="0" t="n">
+      <c r="E314" s="0" t="n">
         <v>31213</v>
-      </c>
-    </row>
-    <row r="314" ht="15.75" customHeight="1" s="4">
-      <c r="B314" s="3" t="inlineStr">
-        <is>
-          <t>LICITACAO</t>
-        </is>
-      </c>
-      <c r="E314" s="3" t="n">
-        <v>31300</v>
       </c>
     </row>
     <row r="315" ht="15.75" customHeight="1" s="4">
       <c r="B315" s="3" t="inlineStr">
         <is>
-          <t>CONTRATOS</t>
+          <t>LICITACAO</t>
         </is>
       </c>
       <c r="E315" s="3" t="n">
-        <v>31400</v>
+        <v>31300</v>
       </c>
     </row>
     <row r="316" ht="15.75" customHeight="1" s="4">
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>EXECUCAO FINANCEIRA</t>
+          <t>CONTRATOS</t>
         </is>
       </c>
       <c r="E316" s="3" t="n">
-        <v>31500</v>
+        <v>31400</v>
       </c>
     </row>
     <row r="317" ht="15.75" customHeight="1" s="4">
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>CONTABILIDADE</t>
+          <t>EXECUCAO FINANCEIRA</t>
         </is>
       </c>
       <c r="E317" s="3" t="n">
-        <v>31600</v>
+        <v>31500</v>
       </c>
     </row>
     <row r="318" ht="15.75" customHeight="1" s="4">
       <c r="B318" s="3" t="inlineStr">
         <is>
+          <t>CONTABILIDADE</t>
+        </is>
+      </c>
+      <c r="E318" s="3" t="n">
+        <v>31600</v>
+      </c>
+    </row>
+    <row r="319" ht="15.75" customHeight="1" s="4">
+      <c r="B319" s="3" t="inlineStr">
+        <is>
           <t>TRANSPORTE</t>
         </is>
-      </c>
-    </row>
-    <row r="319" ht="15.75" customHeight="1" s="4">
-      <c r="C319" s="3" t="inlineStr">
-        <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="E319" s="3" t="n">
-        <v>31700</v>
       </c>
     </row>
     <row r="320" ht="15.75" customHeight="1" s="4">
       <c r="C320" s="3" t="inlineStr">
         <is>
-          <t>TRANSPORTE - SALA</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="E320" s="3" t="n">
-        <v>31701</v>
+        <v>31700</v>
       </c>
     </row>
     <row r="321" ht="15.75" customHeight="1" s="4">
       <c r="C321" s="3" t="inlineStr">
         <is>
+          <t>TRANSPORTE - SALA</t>
+        </is>
+      </c>
+      <c r="E321" s="3" t="n">
+        <v>31701</v>
+      </c>
+    </row>
+    <row r="322" ht="15.75" customHeight="1" s="4">
+      <c r="C322" s="3" t="inlineStr">
+        <is>
           <t>TRANSPORTE - GARAGEM</t>
         </is>
       </c>
-      <c r="E321" s="3" t="n">
+      <c r="E322" s="3" t="n">
         <v>31702</v>
       </c>
     </row>
-    <row r="322" ht="15.75" customHeight="1" s="4">
-      <c r="A322" s="3" t="inlineStr">
+    <row r="323" ht="15.75" customHeight="1" s="4">
+      <c r="A323" s="3" t="inlineStr">
         <is>
           <t>DIRETORIA DE EXTENSÃO</t>
         </is>
-      </c>
-    </row>
-    <row r="323" ht="15.75" customHeight="1" s="4">
-      <c r="B323" s="3" t="inlineStr">
-        <is>
-          <t>DIRETORIA DE EXTENSÃO</t>
-        </is>
-      </c>
-      <c r="E323" s="3" t="n">
-        <v>40000</v>
       </c>
     </row>
     <row r="324" ht="15.75" customHeight="1" s="4">
       <c r="B324" s="3" t="inlineStr">
         <is>
-          <t>SARC - SEÇÃO DE ARTE E CULTURA</t>
+          <t>DIRETORIA DE EXTENSÃO</t>
         </is>
       </c>
       <c r="E324" s="3" t="n">
-        <v>41000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="325" ht="15.75" customHeight="1" s="4">
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>SEÇÃO DE ESTÁGIO</t>
+          <t>SARC - SEÇÃO DE ARTE E CULTURA</t>
         </is>
       </c>
       <c r="E325" s="3" t="n">
-        <v>42000</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="326" ht="15.75" customHeight="1" s="4">
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>RELAÇÕES INSTITUCIONAIS</t>
+          <t>SEÇÃO DE ESTÁGIO</t>
         </is>
       </c>
       <c r="E326" s="3" t="n">
-        <v>43000</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="327" ht="15.75" customHeight="1" s="4">
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>SEÇÃO DE AÇÕES COMUNITÁRIAS</t>
+          <t>RELAÇÕES INSTITUCIONAIS</t>
         </is>
       </c>
       <c r="E327" s="3" t="n">
-        <v>44000</v>
+        <v>43000</v>
       </c>
     </row>
     <row r="328" ht="15.75" customHeight="1" s="4">
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>SALA PROJETO PARTIU IF</t>
+          <t>SEÇÃO DE AÇÕES COMUNITÁRIAS</t>
         </is>
       </c>
       <c r="E328" s="3" t="n">
-        <v>44001</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="329" ht="15.75" customHeight="1" s="4">
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>SALA DA DIRETORIA DE EXTENSÃO</t>
+          <t>SALA PROJETO PARTIU IF</t>
         </is>
       </c>
       <c r="E329" s="3" t="n">
-        <v>45000</v>
+        <v>44001</v>
       </c>
     </row>
     <row r="330" ht="15.75" customHeight="1" s="4">
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>SALA DE REUNIÃO</t>
+          <t>SALA DA DIRETORIA DE EXTENSÃO</t>
         </is>
       </c>
       <c r="E330" s="3" t="n">
-        <v>46000</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="331" ht="15.75" customHeight="1" s="4">
       <c r="B331" s="3" t="inlineStr">
         <is>
+          <t>SALA DE REUNIÃO</t>
+        </is>
+      </c>
+      <c r="E331" s="3" t="n">
+        <v>46000</v>
+      </c>
+    </row>
+    <row r="332" ht="15.75" customHeight="1" s="4">
+      <c r="B332" s="3" t="inlineStr">
+        <is>
           <t>EMPRESA JUNIOR</t>
         </is>
-      </c>
-    </row>
-    <row r="332" ht="15.75" customHeight="1" s="4">
-      <c r="C332" s="3" t="inlineStr">
-        <is>
-          <t>EMPRESA JUNIOR</t>
-        </is>
-      </c>
-      <c r="E332" s="3" t="n">
-        <v>47000</v>
       </c>
     </row>
     <row r="333" ht="15.75" customHeight="1" s="4">
       <c r="C333" s="3" t="inlineStr">
         <is>
-          <t>EMPRESA JUNIOR AGROECO JR (ANTIGO ALOJAMENTO / BLOCO B / SALA 3)</t>
+          <t>EMPRESA JUNIOR</t>
         </is>
       </c>
       <c r="E333" s="3" t="n">
-        <v>47001</v>
+        <v>47000</v>
       </c>
     </row>
     <row r="334" ht="15.75" customHeight="1" s="4">
       <c r="C334" s="3" t="inlineStr">
         <is>
+          <t>EMPRESA JUNIOR AGROECO JR (ANTIGO ALOJAMENTO / BLOCO B / SALA 3)</t>
+        </is>
+      </c>
+      <c r="E334" s="3" t="n">
+        <v>47001</v>
+      </c>
+    </row>
+    <row r="335" ht="15.75" customHeight="1" s="4">
+      <c r="C335" s="3" t="inlineStr">
+        <is>
           <t>EMPRESA JUNIOR EMCOMP (ANTIGO ALOJAMENTO / BLOCO B / SALA 4)</t>
         </is>
       </c>
-      <c r="E334" s="3" t="n">
+      <c r="E335" s="3" t="n">
         <v>47002</v>
       </c>
     </row>
-    <row r="335" ht="15.75" customHeight="1" s="4">
-      <c r="B335" s="3" t="inlineStr">
+    <row r="336" ht="15.75" customHeight="1" s="4">
+      <c r="B336" s="3" t="inlineStr">
         <is>
           <t>TEATRO (ANTIGO ALOJAMENTO/BLOCO B/SALA 5)</t>
         </is>
       </c>
-      <c r="E335" s="3" t="n">
+      <c r="E336" s="3" t="n">
         <v>48000</v>
       </c>
     </row>
-    <row r="336" ht="15.75" customHeight="1" s="4">
-      <c r="A336" s="3" t="inlineStr">
+    <row r="337" ht="15.75" customHeight="1" s="4">
+      <c r="A337" s="3" t="inlineStr">
         <is>
           <t>DIRETORIA DE PESQUISA E POS-GRADUACAO</t>
         </is>
-      </c>
-    </row>
-    <row r="337" ht="15.75" customHeight="1" s="4">
-      <c r="B337" s="3" t="inlineStr">
-        <is>
-          <t>DIRETORIA DE PESQUISA E POS-GRADUACAO</t>
-        </is>
-      </c>
-      <c r="E337" s="3" t="n">
-        <v>50000</v>
       </c>
     </row>
     <row r="338" ht="15.75" customHeight="1" s="4">
       <c r="B338" s="3" t="inlineStr">
         <is>
+          <t>DIRETORIA DE PESQUISA E POS-GRADUACAO</t>
+        </is>
+      </c>
+      <c r="E338" s="3" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="339" ht="15.75" customHeight="1" s="4">
+      <c r="B339" s="3" t="inlineStr">
+        <is>
           <t>POS-GRADUAÇÃO LATO SENSU</t>
         </is>
-      </c>
-    </row>
-    <row r="339" ht="15.75" customHeight="1" s="4">
-      <c r="C339" s="3" t="inlineStr">
-        <is>
-          <t>ESPECIALIZACAO</t>
-        </is>
-      </c>
-      <c r="E339" s="3" t="n">
-        <v>51000</v>
       </c>
     </row>
     <row r="340" ht="15.75" customHeight="1" s="4">
       <c r="C340" s="3" t="inlineStr">
         <is>
-          <t>ESPECIALIZACAO AGROECOLOGIA</t>
+          <t>ESPECIALIZACAO</t>
         </is>
       </c>
       <c r="E340" s="3" t="n">
-        <v>51100</v>
+        <v>51000</v>
       </c>
     </row>
     <row r="341" ht="15.75" customHeight="1" s="4">
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>ESPECIALIZACAO DESENVOLVIMENTO WEB</t>
+          <t>ESPECIALIZACAO AGROECOLOGIA</t>
         </is>
       </c>
       <c r="E341" s="3" t="n">
-        <v>51200</v>
+        <v>51100</v>
       </c>
     </row>
     <row r="342" ht="15.75" customHeight="1" s="4">
       <c r="C342" s="3" t="inlineStr">
         <is>
+          <t>ESPECIALIZACAO DESENVOLVIMENTO WEB</t>
+        </is>
+      </c>
+      <c r="E342" s="3" t="n">
+        <v>51200</v>
+      </c>
+    </row>
+    <row r="343" ht="15.75" customHeight="1" s="4">
+      <c r="C343" s="3" t="inlineStr">
+        <is>
           <t>ESPECIALIZACAO ENSINO DE MATEMATICA E FISICA</t>
         </is>
       </c>
-      <c r="E342" s="3" t="n">
+      <c r="E343" s="3" t="n">
         <v>51300</v>
       </c>
     </row>
-    <row r="343" ht="15.75" customHeight="1" s="4">
-      <c r="B343" s="3" t="inlineStr">
+    <row r="344" ht="15.75" customHeight="1" s="4">
+      <c r="B344" s="3" t="inlineStr">
         <is>
           <t>MESTRADO</t>
         </is>
-      </c>
-    </row>
-    <row r="344" ht="15.75" customHeight="1" s="4">
-      <c r="C344" s="3" t="inlineStr">
-        <is>
-          <t>MESTRADO</t>
-        </is>
-      </c>
-      <c r="E344" s="3" t="n">
-        <v>52000</v>
       </c>
     </row>
     <row r="345" ht="15.75" customHeight="1" s="4">
       <c r="C345" s="3" t="inlineStr">
         <is>
+          <t>MESTRADO</t>
+        </is>
+      </c>
+      <c r="E345" s="3" t="n">
+        <v>52000</v>
+      </c>
+    </row>
+    <row r="346" ht="15.75" customHeight="1" s="4">
+      <c r="C346" s="3" t="inlineStr">
+        <is>
           <t>MESTRADO PROFEPT</t>
         </is>
-      </c>
-    </row>
-    <row r="346" ht="15.75" customHeight="1" s="4">
-      <c r="D346" s="3" t="inlineStr">
-        <is>
-          <t>MESTRADO PROFEPT</t>
-        </is>
-      </c>
-      <c r="E346" s="3" t="n">
-        <v>52100</v>
       </c>
     </row>
     <row r="347" ht="15.75" customHeight="1" s="4">
       <c r="D347" s="3" t="inlineStr">
         <is>
-          <t>PROFEPT - SALA DA COORDENACAO</t>
+          <t>MESTRADO PROFEPT</t>
         </is>
       </c>
       <c r="E347" s="3" t="n">
-        <v>52101</v>
+        <v>52100</v>
       </c>
     </row>
     <row r="348" ht="15.75" customHeight="1" s="4">
       <c r="D348" s="3" t="inlineStr">
         <is>
+          <t>PROFEPT - SALA DA COORDENACAO</t>
+        </is>
+      </c>
+      <c r="E348" s="3" t="n">
+        <v>52101</v>
+      </c>
+    </row>
+    <row r="349" ht="15.75" customHeight="1" s="4">
+      <c r="D349" s="3" t="inlineStr">
+        <is>
           <t>PROFEPT - SALAS DE AULA</t>
         </is>
       </c>
-      <c r="E348" s="3" t="n">
+      <c r="E349" s="3" t="n">
         <v>52102</v>
-      </c>
-    </row>
-    <row r="349" ht="15.75" customHeight="1" s="4">
-      <c r="C349" s="3" t="inlineStr">
-        <is>
-          <t>MESTRADO PROFISSIONAL NUTRICAO E PRODUCAO ANIMAL</t>
-        </is>
-      </c>
-      <c r="E349" s="3" t="n">
-        <v>52200</v>
       </c>
     </row>
     <row r="350" ht="15.75" customHeight="1" s="4">
       <c r="C350" s="3" t="inlineStr">
         <is>
+          <t>MESTRADO PROFISSIONAL NUTRICAO E PRODUCAO ANIMAL</t>
+        </is>
+      </c>
+      <c r="E350" s="3" t="n">
+        <v>52200</v>
+      </c>
+    </row>
+    <row r="351" ht="15.75" customHeight="1" s="4">
+      <c r="C351" s="3" t="inlineStr">
+        <is>
           <t>MESTRADO PROFISSIONAL ALIMENTOS</t>
         </is>
       </c>
-      <c r="E350" s="3" t="n">
+      <c r="E351" s="3" t="n">
         <v>52300</v>
-      </c>
-    </row>
-    <row r="351" ht="15.75" customHeight="1" s="4">
-      <c r="B351" s="3" t="inlineStr">
-        <is>
-          <t>DOUTORADO</t>
-        </is>
-      </c>
-      <c r="E351" s="3" t="n">
-        <v>53000</v>
       </c>
     </row>
     <row r="352" ht="15.75" customHeight="1" s="4">
       <c r="B352" s="3" t="inlineStr">
         <is>
-          <t>NITTEC</t>
+          <t>DOUTORADO</t>
         </is>
       </c>
       <c r="E352" s="3" t="n">
-        <v>54000</v>
+        <v>53000</v>
       </c>
     </row>
     <row r="353" ht="15.75" customHeight="1" s="4">
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>IF MAKER / NITTEC / IPCA</t>
+          <t>NITTEC</t>
         </is>
       </c>
       <c r="E353" s="3" t="n">
-        <v>54001</v>
+        <v>54000</v>
       </c>
     </row>
     <row r="354" ht="15.75" customHeight="1" s="4">
       <c r="B354" s="3" t="inlineStr">
         <is>
+          <t>IF MAKER / NITTEC / IPCA</t>
+        </is>
+      </c>
+      <c r="E354" s="3" t="n">
+        <v>54001</v>
+      </c>
+    </row>
+    <row r="355" ht="15.75" customHeight="1" s="4">
+      <c r="B355" s="3" t="inlineStr">
+        <is>
           <t>GERENCIA DE PESQUISA</t>
         </is>
       </c>
-      <c r="E354" s="3" t="n">
+      <c r="E355" s="3" t="n">
         <v>55000</v>
       </c>
     </row>
-    <row r="355" ht="15.75" customHeight="1" s="4">
-      <c r="A355" s="3" t="inlineStr">
+    <row r="356" ht="15.75" customHeight="1" s="4">
+      <c r="A356" s="3" t="inlineStr">
         <is>
           <t>DIRETORIA DE DESENVOLVIMENTO INSTITUCIONAL</t>
         </is>
-      </c>
-    </row>
-    <row r="356" ht="15.75" customHeight="1" s="4">
-      <c r="B356" s="3" t="inlineStr">
-        <is>
-          <t>DIRETORIA DE DESENVOLVIMENTO INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="E356" s="3" t="n">
-        <v>60000</v>
       </c>
     </row>
     <row r="357" ht="15.75" customHeight="1" s="4">
       <c r="B357" s="3" t="inlineStr">
         <is>
+          <t>DIRETORIA DE DESENVOLVIMENTO INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E357" s="3" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="358" ht="15.75" customHeight="1" s="4">
+      <c r="B358" s="3" t="inlineStr">
+        <is>
           <t>PREFEITURA</t>
         </is>
-      </c>
-    </row>
-    <row r="358" ht="15.75" customHeight="1" s="4">
-      <c r="C358" s="3" t="inlineStr">
-        <is>
-          <t>PREFEITURA</t>
-        </is>
-      </c>
-      <c r="E358" s="3" t="n">
-        <v>61000</v>
       </c>
     </row>
     <row r="359" ht="15.75" customHeight="1" s="4">
       <c r="C359" s="3" t="inlineStr">
         <is>
-          <t>VIGILANCIA</t>
+          <t>PREFEITURA</t>
         </is>
       </c>
       <c r="E359" s="3" t="n">
-        <v>61100</v>
+        <v>61000</v>
       </c>
     </row>
     <row r="360" ht="15.75" customHeight="1" s="4">
       <c r="C360" s="3" t="inlineStr">
         <is>
-          <t>RECICLAGEM</t>
+          <t>VIGILANCIA</t>
         </is>
       </c>
       <c r="E360" s="3" t="n">
-        <v>61200</v>
+        <v>61100</v>
       </c>
     </row>
     <row r="361" ht="15.75" customHeight="1" s="4">
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>SEÇÃO DE SERVICO DE APOIO</t>
+          <t>RECICLAGEM</t>
         </is>
       </c>
       <c r="E361" s="3" t="n">
-        <v>61300</v>
+        <v>61200</v>
       </c>
     </row>
     <row r="362" ht="15.75" customHeight="1" s="4">
       <c r="C362" s="3" t="inlineStr">
         <is>
-          <t>PREFEITURA - ESTACAO DE TRATAMENTO DE AGUA</t>
+          <t>SEÇÃO DE SERVICO DE APOIO</t>
         </is>
       </c>
       <c r="E362" s="3" t="n">
-        <v>61400</v>
+        <v>61300</v>
       </c>
     </row>
     <row r="363" ht="15.75" customHeight="1" s="4">
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>PREFEITURA - MANUTEN. E DEPOS. MATER.CONSTRU</t>
+          <t>PREFEITURA - ESTACAO DE TRATAMENTO DE AGUA</t>
         </is>
       </c>
       <c r="E363" s="3" t="n">
-        <v>61401</v>
+        <v>61400</v>
       </c>
     </row>
     <row r="364" ht="15.75" customHeight="1" s="4">
       <c r="C364" s="3" t="inlineStr">
         <is>
-          <t>PREFEITURA - SERRALHERIA</t>
+          <t>PREFEITURA - MANUTEN. E DEPOS. MATER.CONSTRU</t>
         </is>
       </c>
       <c r="E364" s="3" t="n">
-        <v>61402</v>
+        <v>61401</v>
       </c>
     </row>
     <row r="365" ht="15.75" customHeight="1" s="4">
       <c r="C365" s="3" t="inlineStr">
         <is>
+          <t>PREFEITURA - SERRALHERIA</t>
+        </is>
+      </c>
+      <c r="E365" s="3" t="n">
+        <v>61402</v>
+      </c>
+    </row>
+    <row r="366" ht="15.75" customHeight="1" s="4">
+      <c r="C366" s="3" t="inlineStr">
+        <is>
           <t>PREFEITURA - CARPINTARIA</t>
         </is>
       </c>
-      <c r="E365" s="3" t="n">
+      <c r="E366" s="3" t="n">
         <v>61403</v>
       </c>
     </row>
-    <row r="366" ht="15.75" customHeight="1" s="4">
-      <c r="B366" s="3" t="inlineStr">
+    <row r="367" ht="15.75" customHeight="1" s="4">
+      <c r="B367" s="3" t="inlineStr">
         <is>
           <t>COORDENACAO GERAL DE PRODUCAO</t>
         </is>
-      </c>
-    </row>
-    <row r="367" ht="15.75" customHeight="1" s="4">
-      <c r="C367" s="3" t="inlineStr">
-        <is>
-          <t>COORDENACAO GERAL DE PRODUCAO</t>
-        </is>
-      </c>
-      <c r="E367" s="3" t="n">
-        <v>62000</v>
       </c>
     </row>
     <row r="368" ht="15.75" customHeight="1" s="4">
       <c r="C368" s="3" t="inlineStr">
         <is>
-          <t>MECANIZACAO AGRICOLA</t>
+          <t>COORDENACAO GERAL DE PRODUCAO</t>
         </is>
       </c>
       <c r="E368" s="3" t="n">
-        <v>62100</v>
+        <v>62000</v>
       </c>
     </row>
     <row r="369" ht="15.75" customHeight="1" s="4">
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>POSTO DE VENDAS</t>
+          <t>MECANIZACAO AGRICOLA</t>
         </is>
       </c>
       <c r="E369" s="3" t="n">
-        <v>62200</v>
+        <v>62100</v>
       </c>
     </row>
     <row r="370" ht="15.75" customHeight="1" s="4">
       <c r="C370" s="3" t="inlineStr">
         <is>
-          <t>SECAO DE PROJETOS E PRODUCAO AGROINDUSTRIAL</t>
+          <t>POSTO DE VENDAS</t>
         </is>
       </c>
       <c r="E370" s="3" t="n">
-        <v>62300</v>
+        <v>62200</v>
       </c>
     </row>
     <row r="371" ht="15.75" customHeight="1" s="4">
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>PADARIA</t>
+          <t>SECAO DE PROJETOS E PRODUCAO AGROINDUSTRIAL</t>
         </is>
       </c>
       <c r="E371" s="3" t="n">
-        <v>62301</v>
+        <v>62300</v>
       </c>
     </row>
     <row r="372" ht="15.75" customHeight="1" s="4">
       <c r="C372" s="3" t="inlineStr">
         <is>
-          <t>FRUTAS</t>
+          <t>PADARIA</t>
         </is>
       </c>
       <c r="E372" s="3" t="n">
-        <v>62302</v>
+        <v>62301</v>
       </c>
     </row>
     <row r="373" ht="15.75" customHeight="1" s="4">
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>CARNES</t>
+          <t>FRUTAS</t>
         </is>
       </c>
       <c r="E373" s="3" t="n">
-        <v>62303</v>
+        <v>62302</v>
       </c>
     </row>
     <row r="374" ht="15.75" customHeight="1" s="4">
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>INDUSTRIAS RURAIS</t>
+          <t>CARNES</t>
         </is>
       </c>
       <c r="E374" s="3" t="n">
-        <v>62304</v>
+        <v>62303</v>
       </c>
     </row>
     <row r="375" ht="15.75" customHeight="1" s="4">
       <c r="C375" s="3" t="inlineStr">
         <is>
-          <t>AGROINDUSTRIA - ESCRITORIO E ALMOXARIFADO</t>
+          <t>INDUSTRIAS RURAIS</t>
         </is>
       </c>
       <c r="E375" s="3" t="n">
-        <v>62305</v>
+        <v>62304</v>
       </c>
     </row>
     <row r="376" ht="15.75" customHeight="1" s="4">
       <c r="C376" s="3" t="inlineStr">
         <is>
-          <t>LATICINIO</t>
+          <t>AGROINDUSTRIA - ESCRITORIO E ALMOXARIFADO</t>
         </is>
       </c>
       <c r="E376" s="3" t="n">
-        <v>62306</v>
+        <v>62305</v>
       </c>
     </row>
     <row r="377" ht="15.75" customHeight="1" s="4">
       <c r="C377" s="3" t="inlineStr">
         <is>
+          <t>LATICINIO</t>
+        </is>
+      </c>
+      <c r="E377" s="3" t="n">
+        <v>62306</v>
+      </c>
+    </row>
+    <row r="378" ht="15.75" customHeight="1" s="4">
+      <c r="C378" s="3" t="inlineStr">
+        <is>
           <t>CALDEIRA</t>
         </is>
       </c>
-      <c r="E377" s="3" t="n">
+      <c r="E378" s="3" t="n">
         <v>62307</v>
       </c>
     </row>
-    <row r="378" ht="15.75" customHeight="1" s="4">
-      <c r="B378" s="3" t="inlineStr">
+    <row r="379" ht="15.75" customHeight="1" s="4">
+      <c r="B379" s="3" t="inlineStr">
         <is>
           <t>GERENCIA DE TECNOLOGIA DA INFORMACAO</t>
         </is>
-      </c>
-    </row>
-    <row r="379" ht="15.75" customHeight="1" s="4">
-      <c r="C379" s="3" t="inlineStr">
-        <is>
-          <t>GERENCIA DE TECNOLOGIA DA INFORMACAO</t>
-        </is>
-      </c>
-      <c r="E379" s="3" t="n">
-        <v>63000</v>
       </c>
     </row>
     <row r="380" ht="15.75" customHeight="1" s="4">
       <c r="C380" s="3" t="inlineStr">
         <is>
+          <t>GERENCIA DE TECNOLOGIA DA INFORMACAO</t>
+        </is>
+      </c>
+      <c r="E380" s="3" t="n">
+        <v>63000</v>
+      </c>
+    </row>
+    <row r="381" ht="15.75" customHeight="1" s="4">
+      <c r="C381" s="3" t="inlineStr">
+        <is>
           <t>TI - DATACENTER</t>
         </is>
       </c>
-      <c r="E380" s="3" t="n">
+      <c r="E381" s="3" t="n">
         <v>63001</v>
       </c>
     </row>
-    <row r="381" ht="15.75" customHeight="1" s="4">
-      <c r="A381" s="3" t="inlineStr">
+    <row r="382" ht="15.75" customHeight="1" s="4">
+      <c r="A382" s="3" t="inlineStr">
         <is>
           <t>DIRETOR GERAL</t>
         </is>
-      </c>
-    </row>
-    <row r="382" ht="15.75" customHeight="1" s="4">
-      <c r="B382" s="3" t="inlineStr">
-        <is>
-          <t>DIRETOR GERAL</t>
-        </is>
-      </c>
-      <c r="E382" s="3" t="n">
-        <v>70000</v>
       </c>
     </row>
     <row r="383" ht="15.75" customHeight="1" s="4">
       <c r="B383" s="3" t="inlineStr">
         <is>
-          <t>EMPRESTIMO DE BENS</t>
+          <t>DIRETOR GERAL</t>
         </is>
       </c>
       <c r="E383" s="3" t="n">
-        <v>70001</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="384" ht="15.75" customHeight="1" s="4">
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>AUDITORIA INTERNA</t>
+          <t>EMPRESTIMO DE BENS</t>
         </is>
       </c>
       <c r="E384" s="3" t="n">
-        <v>70002</v>
+        <v>70001</v>
       </c>
     </row>
     <row r="385" ht="15.75" customHeight="1" s="4">
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>ARQUIVO MORTO / GERAL</t>
+          <t>AUDITORIA INTERNA</t>
         </is>
       </c>
       <c r="E385" s="3" t="n">
-        <v>70003</v>
+        <v>70002</v>
       </c>
     </row>
     <row r="386" ht="15.75" customHeight="1" s="4">
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>CESSAO DE BENS</t>
+          <t>ARQUIVO MORTO / GERAL</t>
         </is>
       </c>
       <c r="E386" s="3" t="n">
-        <v>70004</v>
+        <v>70003</v>
       </c>
     </row>
     <row r="387" ht="15.75" customHeight="1" s="4">
       <c r="B387" s="3" t="inlineStr">
         <is>
-          <t>SALAO NOBRE</t>
+          <t>CESSAO DE BENS</t>
         </is>
       </c>
       <c r="E387" s="3" t="n">
-        <v>70005</v>
+        <v>70004</v>
       </c>
     </row>
     <row r="388" ht="15.75" customHeight="1" s="4">
       <c r="B388" s="3" t="inlineStr">
         <is>
-          <t>GABINETE</t>
+          <t>SALAO NOBRE</t>
         </is>
       </c>
       <c r="E388" s="3" t="n">
-        <v>70006</v>
+        <v>70005</v>
       </c>
     </row>
     <row r="389" ht="15.75" customHeight="1" s="4">
       <c r="B389" s="3" t="inlineStr">
         <is>
-          <t>GESTAO DE PESSOAS</t>
+          <t>GABINETE</t>
         </is>
       </c>
       <c r="E389" s="3" t="n">
-        <v>70007</v>
+        <v>70006</v>
       </c>
     </row>
     <row r="390" ht="15.75" customHeight="1" s="4">
       <c r="B390" s="3" t="inlineStr">
         <is>
+          <t>GESTAO DE PESSOAS</t>
+        </is>
+      </c>
+      <c r="E390" s="3" t="n">
+        <v>70007</v>
+      </c>
+    </row>
+    <row r="391" ht="15.75" customHeight="1" s="4">
+      <c r="B391" s="3" t="inlineStr">
+        <is>
           <t>FUNDACAO</t>
         </is>
-      </c>
-    </row>
-    <row r="391" ht="15.75" customHeight="1" s="4">
-      <c r="C391" s="3" t="inlineStr">
-        <is>
-          <t>FUNDACAO - REFEITORIO</t>
-        </is>
-      </c>
-      <c r="E391" s="3" t="n">
-        <v>70009</v>
       </c>
     </row>
     <row r="392" ht="15.75" customHeight="1" s="4">
       <c r="C392" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 1</t>
+          <t>FUNDACAO - REFEITORIO</t>
         </is>
       </c>
       <c r="E392" s="3" t="n">
-        <v>70011</v>
+        <v>70009</v>
       </c>
     </row>
     <row r="393" ht="15.75" customHeight="1" s="4">
       <c r="C393" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 2</t>
+          <t>FUNDACAO - DORMITORIO 1</t>
         </is>
       </c>
       <c r="E393" s="3" t="n">
-        <v>70012</v>
+        <v>70011</v>
       </c>
     </row>
     <row r="394" ht="15.75" customHeight="1" s="4">
       <c r="C394" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 3</t>
+          <t>FUNDACAO - DORMITORIO 2</t>
         </is>
       </c>
       <c r="E394" s="3" t="n">
-        <v>70013</v>
+        <v>70012</v>
       </c>
     </row>
     <row r="395" ht="15.75" customHeight="1" s="4">
       <c r="C395" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 4</t>
+          <t>FUNDACAO - DORMITORIO 3</t>
         </is>
       </c>
       <c r="E395" s="3" t="n">
-        <v>70014</v>
+        <v>70013</v>
       </c>
     </row>
     <row r="396" ht="15.75" customHeight="1" s="4">
       <c r="C396" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 5</t>
+          <t>FUNDACAO - DORMITORIO 4</t>
         </is>
       </c>
       <c r="E396" s="3" t="n">
-        <v>70015</v>
+        <v>70014</v>
       </c>
     </row>
     <row r="397" ht="15.75" customHeight="1" s="4">
       <c r="C397" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 6</t>
+          <t>FUNDACAO - DORMITORIO 5</t>
         </is>
       </c>
       <c r="E397" s="3" t="n">
-        <v>70016</v>
+        <v>70015</v>
       </c>
     </row>
     <row r="398" ht="15.75" customHeight="1" s="4">
       <c r="C398" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 7</t>
+          <t>FUNDACAO - DORMITORIO 6</t>
         </is>
       </c>
       <c r="E398" s="3" t="n">
-        <v>70017</v>
+        <v>70016</v>
       </c>
     </row>
     <row r="399" ht="15.75" customHeight="1" s="4">
       <c r="C399" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 8</t>
+          <t>FUNDACAO - DORMITORIO 7</t>
         </is>
       </c>
       <c r="E399" s="3" t="n">
-        <v>70018</v>
+        <v>70017</v>
       </c>
     </row>
     <row r="400" ht="15.75" customHeight="1" s="4">
       <c r="C400" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 9</t>
+          <t>FUNDACAO - DORMITORIO 8</t>
         </is>
       </c>
       <c r="E400" s="3" t="n">
-        <v>70019</v>
+        <v>70018</v>
       </c>
     </row>
     <row r="401" ht="15.75" customHeight="1" s="4">
       <c r="C401" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 10</t>
+          <t>FUNDACAO - DORMITORIO 9</t>
         </is>
       </c>
       <c r="E401" s="3" t="n">
-        <v>70020</v>
+        <v>70019</v>
       </c>
     </row>
     <row r="402" ht="15.75" customHeight="1" s="4">
       <c r="C402" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 11</t>
+          <t>FUNDACAO - DORMITORIO 10</t>
         </is>
       </c>
       <c r="E402" s="3" t="n">
-        <v>70021</v>
+        <v>70020</v>
       </c>
     </row>
     <row r="403" ht="15.75" customHeight="1" s="4">
       <c r="C403" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - HALL SEGUNDO ANDAR</t>
+          <t>FUNDACAO - DORMITORIO 11</t>
         </is>
       </c>
       <c r="E403" s="3" t="n">
-        <v>70022</v>
+        <v>70021</v>
       </c>
     </row>
     <row r="404" ht="15.75" customHeight="1" s="4">
       <c r="C404" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - SALA SEGUNDO ANDAR</t>
+          <t>FUNDACAO - HALL SEGUNDO ANDAR</t>
         </is>
       </c>
       <c r="E404" s="3" t="n">
-        <v>70023</v>
+        <v>70022</v>
       </c>
     </row>
     <row r="405" ht="15.75" customHeight="1" s="4">
       <c r="C405" s="3" t="inlineStr">
         <is>
+          <t>FUNDACAO - SALA SEGUNDO ANDAR</t>
+        </is>
+      </c>
+      <c r="E405" s="3" t="n">
+        <v>70023</v>
+      </c>
+    </row>
+    <row r="406" ht="15.75" customHeight="1" s="4">
+      <c r="C406" s="3" t="inlineStr">
+        <is>
           <t>FUNDACAO - ANFITEATRO JARBAS FURTADO</t>
         </is>
       </c>
-      <c r="E405" s="3" t="n">
+      <c r="E406" s="3" t="n">
         <v>70010</v>
-      </c>
-    </row>
-    <row r="406" ht="15.75" customHeight="1" s="4">
-      <c r="B406" s="3" t="inlineStr">
-        <is>
-          <t>CENTRO DE VIVENCIA / CANTINA</t>
-        </is>
-      </c>
-      <c r="E406" s="3" t="n">
-        <v>70024</v>
       </c>
     </row>
     <row r="407" ht="15.75" customHeight="1" s="4">
       <c r="B407" s="3" t="inlineStr">
         <is>
+          <t>CENTRO DE VIVENCIA / CANTINA</t>
+        </is>
+      </c>
+      <c r="E407" s="3" t="n">
+        <v>70024</v>
+      </c>
+    </row>
+    <row r="408" ht="15.75" customHeight="1" s="4">
+      <c r="B408" s="3" t="inlineStr">
+        <is>
           <t>ALOJAMENTO - BLOCO C</t>
         </is>
-      </c>
-    </row>
-    <row r="408" ht="15.75" customHeight="1" s="4">
-      <c r="C408" s="3" t="inlineStr">
-        <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 1</t>
-        </is>
-      </c>
-      <c r="E408" s="3" t="n">
-        <v>70025</v>
       </c>
     </row>
     <row r="409" ht="15.75" customHeight="1" s="4">
       <c r="C409" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 2</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 1</t>
         </is>
       </c>
       <c r="E409" s="3" t="n">
-        <v>70026</v>
+        <v>70025</v>
       </c>
     </row>
     <row r="410" ht="15.75" customHeight="1" s="4">
       <c r="C410" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 3</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 2</t>
         </is>
       </c>
       <c r="E410" s="3" t="n">
-        <v>70027</v>
+        <v>70026</v>
       </c>
     </row>
     <row r="411" ht="15.75" customHeight="1" s="4">
       <c r="C411" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 4</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 3</t>
         </is>
       </c>
       <c r="E411" s="3" t="n">
-        <v>70028</v>
+        <v>70027</v>
       </c>
     </row>
     <row r="412" ht="15.75" customHeight="1" s="4">
       <c r="C412" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 5</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 4</t>
         </is>
       </c>
       <c r="E412" s="3" t="n">
-        <v>70029</v>
+        <v>70028</v>
       </c>
     </row>
     <row r="413" ht="15.75" customHeight="1" s="4">
       <c r="C413" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 6</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 5</t>
         </is>
       </c>
       <c r="E413" s="3" t="n">
-        <v>70030</v>
+        <v>70029</v>
       </c>
     </row>
     <row r="414" ht="15.75" customHeight="1" s="4">
       <c r="C414" s="3" t="inlineStr">
         <is>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 6</t>
+        </is>
+      </c>
+      <c r="E414" s="3" t="n">
+        <v>70030</v>
+      </c>
+    </row>
+    <row r="415" ht="15.75" customHeight="1" s="4">
+      <c r="C415" s="3" t="inlineStr">
+        <is>
           <t>ALOJAMENTO - BLOCO C - QUARTO 7</t>
         </is>
       </c>
-      <c r="E414" s="3" t="n">
+      <c r="E415" s="3" t="n">
         <v>70031</v>
       </c>
     </row>
-    <row r="415" ht="15.75" customHeight="1" s="4">
-      <c r="B415" s="3" t="inlineStr">
+    <row r="416" ht="15.75" customHeight="1" s="4">
+      <c r="B416" s="3" t="inlineStr">
         <is>
           <t>ALOJAMENTO - BLOCO D</t>
         </is>
-      </c>
-    </row>
-    <row r="416" ht="15.75" customHeight="1" s="4">
-      <c r="C416" s="3" t="inlineStr">
-        <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 1</t>
-        </is>
-      </c>
-      <c r="E416" s="3" t="n">
-        <v>70032</v>
       </c>
     </row>
     <row r="417" ht="15.75" customHeight="1" s="4">
       <c r="C417" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 2</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 1</t>
         </is>
       </c>
       <c r="E417" s="3" t="n">
-        <v>70033</v>
+        <v>70032</v>
       </c>
     </row>
     <row r="418" ht="15.75" customHeight="1" s="4">
       <c r="C418" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 3</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 2</t>
         </is>
       </c>
       <c r="E418" s="3" t="n">
-        <v>70034</v>
+        <v>70033</v>
       </c>
     </row>
     <row r="419" ht="15.75" customHeight="1" s="4">
       <c r="C419" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 4</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 3</t>
         </is>
       </c>
       <c r="E419" s="3" t="n">
-        <v>70035</v>
+        <v>70034</v>
       </c>
     </row>
     <row r="420" ht="15.75" customHeight="1" s="4">
       <c r="C420" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 5</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 4</t>
         </is>
       </c>
       <c r="E420" s="3" t="n">
-        <v>70036</v>
+        <v>70035</v>
       </c>
     </row>
     <row r="421" ht="15.75" customHeight="1" s="4">
       <c r="C421" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 6</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 5</t>
         </is>
       </c>
       <c r="E421" s="3" t="n">
-        <v>70037</v>
+        <v>70036</v>
       </c>
     </row>
     <row r="422" ht="15.75" customHeight="1" s="4">
       <c r="C422" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 7</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 6</t>
         </is>
       </c>
       <c r="E422" s="3" t="n">
-        <v>70038</v>
+        <v>70037</v>
       </c>
     </row>
     <row r="423" ht="15.75" customHeight="1" s="4">
       <c r="C423" s="3" t="inlineStr">
         <is>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 7</t>
+        </is>
+      </c>
+      <c r="E423" s="3" t="n">
+        <v>70038</v>
+      </c>
+    </row>
+    <row r="424" ht="15.75" customHeight="1" s="4">
+      <c r="C424" s="3" t="inlineStr">
+        <is>
           <t>ALOJAMENTO - GALPAO / DEPOSITO</t>
         </is>
       </c>
-      <c r="E423" s="3" t="n">
+      <c r="E424" s="3" t="n">
         <v>70039</v>
-      </c>
-    </row>
-    <row r="424" ht="15.75" customHeight="1" s="4">
-      <c r="B424" s="0" t="inlineStr">
-        <is>
-          <t>SALA WEB RADIO (ALOJAMENTO / BLOCO B / SALA 1)</t>
-        </is>
-      </c>
-      <c r="E424" s="0" t="n">
-        <v>70040</v>
       </c>
     </row>
     <row r="425" ht="15.75" customHeight="1" s="4">
       <c r="B425" s="0" t="inlineStr">
         <is>
+          <t>SALA WEB RADIO (ALOJAMENTO / BLOCO B / SALA 1)</t>
+        </is>
+      </c>
+      <c r="E425" s="0" t="n">
+        <v>70040</v>
+      </c>
+    </row>
+    <row r="426" ht="15.75" customHeight="1" s="4">
+      <c r="B426" s="0" t="inlineStr">
+        <is>
           <t>CAPELA / IGREJINHA</t>
         </is>
       </c>
-      <c r="E425" s="0" t="n">
+      <c r="E426" s="0" t="n">
         <v>70041</v>
       </c>
     </row>
-    <row r="426" ht="15.75" customHeight="1" s="4">
-      <c r="B426" s="3" t="inlineStr">
+    <row r="427" ht="15.75" customHeight="1" s="4">
+      <c r="B427" s="3" t="inlineStr">
         <is>
           <t>COMUNICACAO</t>
         </is>
-      </c>
-    </row>
-    <row r="427" ht="15.75" customHeight="1" s="4">
-      <c r="C427" s="3" t="inlineStr">
-        <is>
-          <t>COMUNICACAO</t>
-        </is>
-      </c>
-      <c r="E427" s="3" t="n">
-        <v>71000</v>
       </c>
     </row>
     <row r="428" ht="15.75" customHeight="1" s="4">
       <c r="C428" s="3" t="inlineStr">
         <is>
-          <t>SALA DA COMUNICACAO - FUNDACAO</t>
+          <t>COMUNICACAO</t>
         </is>
       </c>
       <c r="E428" s="3" t="n">
-        <v>71002</v>
+        <v>71000</v>
       </c>
     </row>
     <row r="429" ht="15.75" customHeight="1" s="4">
       <c r="C429" s="3" t="inlineStr">
         <is>
+          <t>SALA DA COMUNICACAO - FUNDACAO</t>
+        </is>
+      </c>
+      <c r="E429" s="3" t="n">
+        <v>71002</v>
+      </c>
+    </row>
+    <row r="430" ht="15.75" customHeight="1" s="4">
+      <c r="C430" s="3" t="inlineStr">
+        <is>
           <t>SALA DA COMUNICACAO - PREDIO ADMINISTRATIVO</t>
         </is>
       </c>
-      <c r="E429" s="3" t="n">
+      <c r="E430" s="3" t="n">
         <v>71001</v>
       </c>
     </row>
-    <row r="430" ht="15.75" customHeight="1" s="4"/>
     <row r="431" ht="15.75" customHeight="1" s="4"/>
     <row r="432" ht="15.75" customHeight="1" s="4"/>
     <row r="433" ht="15.75" customHeight="1" s="4"/>

</xml_diff>

<commit_message>
Inclui 70008 CASA DOS INSTRUMENTOS MUSICAIS / CASA DO RAMON
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
+++ b/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
@@ -341,7 +341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E430"/>
+  <dimension ref="A1:E431"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="52" customWidth="1" style="4" min="1" max="1"/>
@@ -3005,12 +3005,12 @@
       </c>
     </row>
     <row r="272" ht="15.75" customHeight="1" s="4">
-      <c r="C272" t="inlineStr">
+      <c r="C272" s="0" t="inlineStr">
         <is>
           <t>LABORATORIO DE ANALISE BIOMECANICA DO MOVIMENTO HUMANO</t>
         </is>
       </c>
-      <c r="E272" t="n">
+      <c r="E272" s="0" t="n">
         <v>26815</v>
       </c>
     </row>
@@ -4141,394 +4141,403 @@
       </c>
     </row>
     <row r="391" ht="15.75" customHeight="1" s="4">
-      <c r="B391" s="3" t="inlineStr">
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>CASA DOS INSTRUMENTOS MUSICAIS / CASA DO RAMON</t>
+        </is>
+      </c>
+      <c r="E391" t="n">
+        <v>70008</v>
+      </c>
+    </row>
+    <row r="392" ht="15.75" customHeight="1" s="4">
+      <c r="B392" s="3" t="inlineStr">
         <is>
           <t>FUNDACAO</t>
         </is>
-      </c>
-    </row>
-    <row r="392" ht="15.75" customHeight="1" s="4">
-      <c r="C392" s="3" t="inlineStr">
-        <is>
-          <t>FUNDACAO - REFEITORIO</t>
-        </is>
-      </c>
-      <c r="E392" s="3" t="n">
-        <v>70009</v>
       </c>
     </row>
     <row r="393" ht="15.75" customHeight="1" s="4">
       <c r="C393" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 1</t>
+          <t>FUNDACAO - REFEITORIO</t>
         </is>
       </c>
       <c r="E393" s="3" t="n">
-        <v>70011</v>
+        <v>70009</v>
       </c>
     </row>
     <row r="394" ht="15.75" customHeight="1" s="4">
       <c r="C394" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 2</t>
+          <t>FUNDACAO - DORMITORIO 1</t>
         </is>
       </c>
       <c r="E394" s="3" t="n">
-        <v>70012</v>
+        <v>70011</v>
       </c>
     </row>
     <row r="395" ht="15.75" customHeight="1" s="4">
       <c r="C395" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 3</t>
+          <t>FUNDACAO - DORMITORIO 2</t>
         </is>
       </c>
       <c r="E395" s="3" t="n">
-        <v>70013</v>
+        <v>70012</v>
       </c>
     </row>
     <row r="396" ht="15.75" customHeight="1" s="4">
       <c r="C396" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 4</t>
+          <t>FUNDACAO - DORMITORIO 3</t>
         </is>
       </c>
       <c r="E396" s="3" t="n">
-        <v>70014</v>
+        <v>70013</v>
       </c>
     </row>
     <row r="397" ht="15.75" customHeight="1" s="4">
       <c r="C397" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 5</t>
+          <t>FUNDACAO - DORMITORIO 4</t>
         </is>
       </c>
       <c r="E397" s="3" t="n">
-        <v>70015</v>
+        <v>70014</v>
       </c>
     </row>
     <row r="398" ht="15.75" customHeight="1" s="4">
       <c r="C398" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 6</t>
+          <t>FUNDACAO - DORMITORIO 5</t>
         </is>
       </c>
       <c r="E398" s="3" t="n">
-        <v>70016</v>
+        <v>70015</v>
       </c>
     </row>
     <row r="399" ht="15.75" customHeight="1" s="4">
       <c r="C399" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 7</t>
+          <t>FUNDACAO - DORMITORIO 6</t>
         </is>
       </c>
       <c r="E399" s="3" t="n">
-        <v>70017</v>
+        <v>70016</v>
       </c>
     </row>
     <row r="400" ht="15.75" customHeight="1" s="4">
       <c r="C400" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 8</t>
+          <t>FUNDACAO - DORMITORIO 7</t>
         </is>
       </c>
       <c r="E400" s="3" t="n">
-        <v>70018</v>
+        <v>70017</v>
       </c>
     </row>
     <row r="401" ht="15.75" customHeight="1" s="4">
       <c r="C401" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 9</t>
+          <t>FUNDACAO - DORMITORIO 8</t>
         </is>
       </c>
       <c r="E401" s="3" t="n">
-        <v>70019</v>
+        <v>70018</v>
       </c>
     </row>
     <row r="402" ht="15.75" customHeight="1" s="4">
       <c r="C402" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 10</t>
+          <t>FUNDACAO - DORMITORIO 9</t>
         </is>
       </c>
       <c r="E402" s="3" t="n">
-        <v>70020</v>
+        <v>70019</v>
       </c>
     </row>
     <row r="403" ht="15.75" customHeight="1" s="4">
       <c r="C403" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 11</t>
+          <t>FUNDACAO - DORMITORIO 10</t>
         </is>
       </c>
       <c r="E403" s="3" t="n">
-        <v>70021</v>
+        <v>70020</v>
       </c>
     </row>
     <row r="404" ht="15.75" customHeight="1" s="4">
       <c r="C404" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - HALL SEGUNDO ANDAR</t>
+          <t>FUNDACAO - DORMITORIO 11</t>
         </is>
       </c>
       <c r="E404" s="3" t="n">
-        <v>70022</v>
+        <v>70021</v>
       </c>
     </row>
     <row r="405" ht="15.75" customHeight="1" s="4">
       <c r="C405" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - SALA SEGUNDO ANDAR</t>
+          <t>FUNDACAO - HALL SEGUNDO ANDAR</t>
         </is>
       </c>
       <c r="E405" s="3" t="n">
-        <v>70023</v>
+        <v>70022</v>
       </c>
     </row>
     <row r="406" ht="15.75" customHeight="1" s="4">
       <c r="C406" s="3" t="inlineStr">
         <is>
+          <t>FUNDACAO - SALA SEGUNDO ANDAR</t>
+        </is>
+      </c>
+      <c r="E406" s="3" t="n">
+        <v>70023</v>
+      </c>
+    </row>
+    <row r="407" ht="15.75" customHeight="1" s="4">
+      <c r="C407" s="3" t="inlineStr">
+        <is>
           <t>FUNDACAO - ANFITEATRO JARBAS FURTADO</t>
         </is>
       </c>
-      <c r="E406" s="3" t="n">
+      <c r="E407" s="3" t="n">
         <v>70010</v>
-      </c>
-    </row>
-    <row r="407" ht="15.75" customHeight="1" s="4">
-      <c r="B407" s="3" t="inlineStr">
-        <is>
-          <t>CENTRO DE VIVENCIA / CANTINA</t>
-        </is>
-      </c>
-      <c r="E407" s="3" t="n">
-        <v>70024</v>
       </c>
     </row>
     <row r="408" ht="15.75" customHeight="1" s="4">
       <c r="B408" s="3" t="inlineStr">
         <is>
+          <t>CENTRO DE VIVENCIA / CANTINA</t>
+        </is>
+      </c>
+      <c r="E408" s="3" t="n">
+        <v>70024</v>
+      </c>
+    </row>
+    <row r="409" ht="15.75" customHeight="1" s="4">
+      <c r="B409" s="3" t="inlineStr">
+        <is>
           <t>ALOJAMENTO - BLOCO C</t>
         </is>
-      </c>
-    </row>
-    <row r="409" ht="15.75" customHeight="1" s="4">
-      <c r="C409" s="3" t="inlineStr">
-        <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 1</t>
-        </is>
-      </c>
-      <c r="E409" s="3" t="n">
-        <v>70025</v>
       </c>
     </row>
     <row r="410" ht="15.75" customHeight="1" s="4">
       <c r="C410" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 2</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 1</t>
         </is>
       </c>
       <c r="E410" s="3" t="n">
-        <v>70026</v>
+        <v>70025</v>
       </c>
     </row>
     <row r="411" ht="15.75" customHeight="1" s="4">
       <c r="C411" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 3</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 2</t>
         </is>
       </c>
       <c r="E411" s="3" t="n">
-        <v>70027</v>
+        <v>70026</v>
       </c>
     </row>
     <row r="412" ht="15.75" customHeight="1" s="4">
       <c r="C412" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 4</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 3</t>
         </is>
       </c>
       <c r="E412" s="3" t="n">
-        <v>70028</v>
+        <v>70027</v>
       </c>
     </row>
     <row r="413" ht="15.75" customHeight="1" s="4">
       <c r="C413" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 5</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 4</t>
         </is>
       </c>
       <c r="E413" s="3" t="n">
-        <v>70029</v>
+        <v>70028</v>
       </c>
     </row>
     <row r="414" ht="15.75" customHeight="1" s="4">
       <c r="C414" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 6</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 5</t>
         </is>
       </c>
       <c r="E414" s="3" t="n">
-        <v>70030</v>
+        <v>70029</v>
       </c>
     </row>
     <row r="415" ht="15.75" customHeight="1" s="4">
       <c r="C415" s="3" t="inlineStr">
         <is>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 6</t>
+        </is>
+      </c>
+      <c r="E415" s="3" t="n">
+        <v>70030</v>
+      </c>
+    </row>
+    <row r="416" ht="15.75" customHeight="1" s="4">
+      <c r="C416" s="3" t="inlineStr">
+        <is>
           <t>ALOJAMENTO - BLOCO C - QUARTO 7</t>
         </is>
       </c>
-      <c r="E415" s="3" t="n">
+      <c r="E416" s="3" t="n">
         <v>70031</v>
       </c>
     </row>
-    <row r="416" ht="15.75" customHeight="1" s="4">
-      <c r="B416" s="3" t="inlineStr">
+    <row r="417" ht="15.75" customHeight="1" s="4">
+      <c r="B417" s="3" t="inlineStr">
         <is>
           <t>ALOJAMENTO - BLOCO D</t>
         </is>
-      </c>
-    </row>
-    <row r="417" ht="15.75" customHeight="1" s="4">
-      <c r="C417" s="3" t="inlineStr">
-        <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 1</t>
-        </is>
-      </c>
-      <c r="E417" s="3" t="n">
-        <v>70032</v>
       </c>
     </row>
     <row r="418" ht="15.75" customHeight="1" s="4">
       <c r="C418" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 2</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 1</t>
         </is>
       </c>
       <c r="E418" s="3" t="n">
-        <v>70033</v>
+        <v>70032</v>
       </c>
     </row>
     <row r="419" ht="15.75" customHeight="1" s="4">
       <c r="C419" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 3</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 2</t>
         </is>
       </c>
       <c r="E419" s="3" t="n">
-        <v>70034</v>
+        <v>70033</v>
       </c>
     </row>
     <row r="420" ht="15.75" customHeight="1" s="4">
       <c r="C420" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 4</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 3</t>
         </is>
       </c>
       <c r="E420" s="3" t="n">
-        <v>70035</v>
+        <v>70034</v>
       </c>
     </row>
     <row r="421" ht="15.75" customHeight="1" s="4">
       <c r="C421" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 5</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 4</t>
         </is>
       </c>
       <c r="E421" s="3" t="n">
-        <v>70036</v>
+        <v>70035</v>
       </c>
     </row>
     <row r="422" ht="15.75" customHeight="1" s="4">
       <c r="C422" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 6</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 5</t>
         </is>
       </c>
       <c r="E422" s="3" t="n">
-        <v>70037</v>
+        <v>70036</v>
       </c>
     </row>
     <row r="423" ht="15.75" customHeight="1" s="4">
       <c r="C423" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 7</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 6</t>
         </is>
       </c>
       <c r="E423" s="3" t="n">
-        <v>70038</v>
+        <v>70037</v>
       </c>
     </row>
     <row r="424" ht="15.75" customHeight="1" s="4">
       <c r="C424" s="3" t="inlineStr">
         <is>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 7</t>
+        </is>
+      </c>
+      <c r="E424" s="3" t="n">
+        <v>70038</v>
+      </c>
+    </row>
+    <row r="425" ht="15.75" customHeight="1" s="4">
+      <c r="C425" s="3" t="inlineStr">
+        <is>
           <t>ALOJAMENTO - GALPAO / DEPOSITO</t>
         </is>
       </c>
-      <c r="E424" s="3" t="n">
+      <c r="E425" s="3" t="n">
         <v>70039</v>
-      </c>
-    </row>
-    <row r="425" ht="15.75" customHeight="1" s="4">
-      <c r="B425" s="0" t="inlineStr">
-        <is>
-          <t>SALA WEB RADIO (ALOJAMENTO / BLOCO B / SALA 1)</t>
-        </is>
-      </c>
-      <c r="E425" s="0" t="n">
-        <v>70040</v>
       </c>
     </row>
     <row r="426" ht="15.75" customHeight="1" s="4">
       <c r="B426" s="0" t="inlineStr">
         <is>
+          <t>SALA WEB RADIO (ALOJAMENTO / BLOCO B / SALA 1)</t>
+        </is>
+      </c>
+      <c r="E426" s="0" t="n">
+        <v>70040</v>
+      </c>
+    </row>
+    <row r="427" ht="15.75" customHeight="1" s="4">
+      <c r="B427" s="0" t="inlineStr">
+        <is>
           <t>CAPELA / IGREJINHA</t>
         </is>
       </c>
-      <c r="E426" s="0" t="n">
+      <c r="E427" s="0" t="n">
         <v>70041</v>
       </c>
     </row>
-    <row r="427" ht="15.75" customHeight="1" s="4">
-      <c r="B427" s="3" t="inlineStr">
+    <row r="428" ht="15.75" customHeight="1" s="4">
+      <c r="B428" s="3" t="inlineStr">
         <is>
           <t>COMUNICACAO</t>
         </is>
-      </c>
-    </row>
-    <row r="428" ht="15.75" customHeight="1" s="4">
-      <c r="C428" s="3" t="inlineStr">
-        <is>
-          <t>COMUNICACAO</t>
-        </is>
-      </c>
-      <c r="E428" s="3" t="n">
-        <v>71000</v>
       </c>
     </row>
     <row r="429" ht="15.75" customHeight="1" s="4">
       <c r="C429" s="3" t="inlineStr">
         <is>
-          <t>SALA DA COMUNICACAO - FUNDACAO</t>
+          <t>COMUNICACAO</t>
         </is>
       </c>
       <c r="E429" s="3" t="n">
-        <v>71002</v>
+        <v>71000</v>
       </c>
     </row>
     <row r="430" ht="15.75" customHeight="1" s="4">
       <c r="C430" s="3" t="inlineStr">
         <is>
+          <t>SALA DA COMUNICACAO - FUNDACAO</t>
+        </is>
+      </c>
+      <c r="E430" s="3" t="n">
+        <v>71002</v>
+      </c>
+    </row>
+    <row r="431" ht="15.75" customHeight="1" s="4">
+      <c r="C431" s="3" t="inlineStr">
+        <is>
           <t>SALA DA COMUNICACAO - PREDIO ADMINISTRATIVO</t>
         </is>
       </c>
-      <c r="E430" s="3" t="n">
+      <c r="E431" s="3" t="n">
         <v>71001</v>
       </c>
     </row>
-    <row r="431" ht="15.75" customHeight="1" s="4"/>
     <row r="432" ht="15.75" customHeight="1" s="4"/>
     <row r="433" ht="15.75" customHeight="1" s="4"/>
     <row r="434" ht="15.75" customHeight="1" s="4"/>

</xml_diff>

<commit_message>
Inclui 31214 PATRIMONIO - RECLASSIFICACAO MATERIAL DE CONSUMO
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
+++ b/CODIGOS_CENTRO_DE_CUSTO_SISERGE_2025_CORRIGIDA.xlsx
@@ -341,7 +341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E431"/>
+  <dimension ref="A1:E432"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="52" customWidth="1" style="4" min="1" max="1"/>
@@ -3417,1128 +3417,1137 @@
       </c>
     </row>
     <row r="315" ht="15.75" customHeight="1" s="4">
-      <c r="B315" s="3" t="inlineStr">
-        <is>
-          <t>LICITACAO</t>
-        </is>
-      </c>
-      <c r="E315" s="3" t="n">
-        <v>31300</v>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>PATRIMONIO - RECLASSIFICACAO MATERIAL DE CONSUMO</t>
+        </is>
+      </c>
+      <c r="E315" t="n">
+        <v>31214</v>
       </c>
     </row>
     <row r="316" ht="15.75" customHeight="1" s="4">
       <c r="B316" s="3" t="inlineStr">
         <is>
-          <t>CONTRATOS</t>
+          <t>LICITACAO</t>
         </is>
       </c>
       <c r="E316" s="3" t="n">
-        <v>31400</v>
+        <v>31300</v>
       </c>
     </row>
     <row r="317" ht="15.75" customHeight="1" s="4">
       <c r="B317" s="3" t="inlineStr">
         <is>
-          <t>EXECUCAO FINANCEIRA</t>
+          <t>CONTRATOS</t>
         </is>
       </c>
       <c r="E317" s="3" t="n">
-        <v>31500</v>
+        <v>31400</v>
       </c>
     </row>
     <row r="318" ht="15.75" customHeight="1" s="4">
       <c r="B318" s="3" t="inlineStr">
         <is>
-          <t>CONTABILIDADE</t>
+          <t>EXECUCAO FINANCEIRA</t>
         </is>
       </c>
       <c r="E318" s="3" t="n">
-        <v>31600</v>
+        <v>31500</v>
       </c>
     </row>
     <row r="319" ht="15.75" customHeight="1" s="4">
       <c r="B319" s="3" t="inlineStr">
         <is>
+          <t>CONTABILIDADE</t>
+        </is>
+      </c>
+      <c r="E319" s="3" t="n">
+        <v>31600</v>
+      </c>
+    </row>
+    <row r="320" ht="15.75" customHeight="1" s="4">
+      <c r="B320" s="3" t="inlineStr">
+        <is>
           <t>TRANSPORTE</t>
         </is>
-      </c>
-    </row>
-    <row r="320" ht="15.75" customHeight="1" s="4">
-      <c r="C320" s="3" t="inlineStr">
-        <is>
-          <t>TRANSPORTE</t>
-        </is>
-      </c>
-      <c r="E320" s="3" t="n">
-        <v>31700</v>
       </c>
     </row>
     <row r="321" ht="15.75" customHeight="1" s="4">
       <c r="C321" s="3" t="inlineStr">
         <is>
-          <t>TRANSPORTE - SALA</t>
+          <t>TRANSPORTE</t>
         </is>
       </c>
       <c r="E321" s="3" t="n">
-        <v>31701</v>
+        <v>31700</v>
       </c>
     </row>
     <row r="322" ht="15.75" customHeight="1" s="4">
       <c r="C322" s="3" t="inlineStr">
         <is>
+          <t>TRANSPORTE - SALA</t>
+        </is>
+      </c>
+      <c r="E322" s="3" t="n">
+        <v>31701</v>
+      </c>
+    </row>
+    <row r="323" ht="15.75" customHeight="1" s="4">
+      <c r="C323" s="3" t="inlineStr">
+        <is>
           <t>TRANSPORTE - GARAGEM</t>
         </is>
       </c>
-      <c r="E322" s="3" t="n">
+      <c r="E323" s="3" t="n">
         <v>31702</v>
       </c>
     </row>
-    <row r="323" ht="15.75" customHeight="1" s="4">
-      <c r="A323" s="3" t="inlineStr">
+    <row r="324" ht="15.75" customHeight="1" s="4">
+      <c r="A324" s="3" t="inlineStr">
         <is>
           <t>DIRETORIA DE EXTENSÃO</t>
         </is>
-      </c>
-    </row>
-    <row r="324" ht="15.75" customHeight="1" s="4">
-      <c r="B324" s="3" t="inlineStr">
-        <is>
-          <t>DIRETORIA DE EXTENSÃO</t>
-        </is>
-      </c>
-      <c r="E324" s="3" t="n">
-        <v>40000</v>
       </c>
     </row>
     <row r="325" ht="15.75" customHeight="1" s="4">
       <c r="B325" s="3" t="inlineStr">
         <is>
-          <t>SARC - SEÇÃO DE ARTE E CULTURA</t>
+          <t>DIRETORIA DE EXTENSÃO</t>
         </is>
       </c>
       <c r="E325" s="3" t="n">
-        <v>41000</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="326" ht="15.75" customHeight="1" s="4">
       <c r="B326" s="3" t="inlineStr">
         <is>
-          <t>SEÇÃO DE ESTÁGIO</t>
+          <t>SARC - SEÇÃO DE ARTE E CULTURA</t>
         </is>
       </c>
       <c r="E326" s="3" t="n">
-        <v>42000</v>
+        <v>41000</v>
       </c>
     </row>
     <row r="327" ht="15.75" customHeight="1" s="4">
       <c r="B327" s="3" t="inlineStr">
         <is>
-          <t>RELAÇÕES INSTITUCIONAIS</t>
+          <t>SEÇÃO DE ESTÁGIO</t>
         </is>
       </c>
       <c r="E327" s="3" t="n">
-        <v>43000</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="328" ht="15.75" customHeight="1" s="4">
       <c r="B328" s="3" t="inlineStr">
         <is>
-          <t>SEÇÃO DE AÇÕES COMUNITÁRIAS</t>
+          <t>RELAÇÕES INSTITUCIONAIS</t>
         </is>
       </c>
       <c r="E328" s="3" t="n">
-        <v>44000</v>
+        <v>43000</v>
       </c>
     </row>
     <row r="329" ht="15.75" customHeight="1" s="4">
       <c r="B329" s="3" t="inlineStr">
         <is>
-          <t>SALA PROJETO PARTIU IF</t>
+          <t>SEÇÃO DE AÇÕES COMUNITÁRIAS</t>
         </is>
       </c>
       <c r="E329" s="3" t="n">
-        <v>44001</v>
+        <v>44000</v>
       </c>
     </row>
     <row r="330" ht="15.75" customHeight="1" s="4">
       <c r="B330" s="3" t="inlineStr">
         <is>
-          <t>SALA DA DIRETORIA DE EXTENSÃO</t>
+          <t>SALA PROJETO PARTIU IF</t>
         </is>
       </c>
       <c r="E330" s="3" t="n">
-        <v>45000</v>
+        <v>44001</v>
       </c>
     </row>
     <row r="331" ht="15.75" customHeight="1" s="4">
       <c r="B331" s="3" t="inlineStr">
         <is>
-          <t>SALA DE REUNIÃO</t>
+          <t>SALA DA DIRETORIA DE EXTENSÃO</t>
         </is>
       </c>
       <c r="E331" s="3" t="n">
-        <v>46000</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="332" ht="15.75" customHeight="1" s="4">
       <c r="B332" s="3" t="inlineStr">
         <is>
+          <t>SALA DE REUNIÃO</t>
+        </is>
+      </c>
+      <c r="E332" s="3" t="n">
+        <v>46000</v>
+      </c>
+    </row>
+    <row r="333" ht="15.75" customHeight="1" s="4">
+      <c r="B333" s="3" t="inlineStr">
+        <is>
           <t>EMPRESA JUNIOR</t>
         </is>
-      </c>
-    </row>
-    <row r="333" ht="15.75" customHeight="1" s="4">
-      <c r="C333" s="3" t="inlineStr">
-        <is>
-          <t>EMPRESA JUNIOR</t>
-        </is>
-      </c>
-      <c r="E333" s="3" t="n">
-        <v>47000</v>
       </c>
     </row>
     <row r="334" ht="15.75" customHeight="1" s="4">
       <c r="C334" s="3" t="inlineStr">
         <is>
-          <t>EMPRESA JUNIOR AGROECO JR (ANTIGO ALOJAMENTO / BLOCO B / SALA 3)</t>
+          <t>EMPRESA JUNIOR</t>
         </is>
       </c>
       <c r="E334" s="3" t="n">
-        <v>47001</v>
+        <v>47000</v>
       </c>
     </row>
     <row r="335" ht="15.75" customHeight="1" s="4">
       <c r="C335" s="3" t="inlineStr">
         <is>
+          <t>EMPRESA JUNIOR AGROECO JR (ANTIGO ALOJAMENTO / BLOCO B / SALA 3)</t>
+        </is>
+      </c>
+      <c r="E335" s="3" t="n">
+        <v>47001</v>
+      </c>
+    </row>
+    <row r="336" ht="15.75" customHeight="1" s="4">
+      <c r="C336" s="3" t="inlineStr">
+        <is>
           <t>EMPRESA JUNIOR EMCOMP (ANTIGO ALOJAMENTO / BLOCO B / SALA 4)</t>
         </is>
       </c>
-      <c r="E335" s="3" t="n">
+      <c r="E336" s="3" t="n">
         <v>47002</v>
       </c>
     </row>
-    <row r="336" ht="15.75" customHeight="1" s="4">
-      <c r="B336" s="3" t="inlineStr">
+    <row r="337" ht="15.75" customHeight="1" s="4">
+      <c r="B337" s="3" t="inlineStr">
         <is>
           <t>TEATRO (ANTIGO ALOJAMENTO/BLOCO B/SALA 5)</t>
         </is>
       </c>
-      <c r="E336" s="3" t="n">
+      <c r="E337" s="3" t="n">
         <v>48000</v>
       </c>
     </row>
-    <row r="337" ht="15.75" customHeight="1" s="4">
-      <c r="A337" s="3" t="inlineStr">
+    <row r="338" ht="15.75" customHeight="1" s="4">
+      <c r="A338" s="3" t="inlineStr">
         <is>
           <t>DIRETORIA DE PESQUISA E POS-GRADUACAO</t>
         </is>
-      </c>
-    </row>
-    <row r="338" ht="15.75" customHeight="1" s="4">
-      <c r="B338" s="3" t="inlineStr">
-        <is>
-          <t>DIRETORIA DE PESQUISA E POS-GRADUACAO</t>
-        </is>
-      </c>
-      <c r="E338" s="3" t="n">
-        <v>50000</v>
       </c>
     </row>
     <row r="339" ht="15.75" customHeight="1" s="4">
       <c r="B339" s="3" t="inlineStr">
         <is>
+          <t>DIRETORIA DE PESQUISA E POS-GRADUACAO</t>
+        </is>
+      </c>
+      <c r="E339" s="3" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="340" ht="15.75" customHeight="1" s="4">
+      <c r="B340" s="3" t="inlineStr">
+        <is>
           <t>POS-GRADUAÇÃO LATO SENSU</t>
         </is>
-      </c>
-    </row>
-    <row r="340" ht="15.75" customHeight="1" s="4">
-      <c r="C340" s="3" t="inlineStr">
-        <is>
-          <t>ESPECIALIZACAO</t>
-        </is>
-      </c>
-      <c r="E340" s="3" t="n">
-        <v>51000</v>
       </c>
     </row>
     <row r="341" ht="15.75" customHeight="1" s="4">
       <c r="C341" s="3" t="inlineStr">
         <is>
-          <t>ESPECIALIZACAO AGROECOLOGIA</t>
+          <t>ESPECIALIZACAO</t>
         </is>
       </c>
       <c r="E341" s="3" t="n">
-        <v>51100</v>
+        <v>51000</v>
       </c>
     </row>
     <row r="342" ht="15.75" customHeight="1" s="4">
       <c r="C342" s="3" t="inlineStr">
         <is>
-          <t>ESPECIALIZACAO DESENVOLVIMENTO WEB</t>
+          <t>ESPECIALIZACAO AGROECOLOGIA</t>
         </is>
       </c>
       <c r="E342" s="3" t="n">
-        <v>51200</v>
+        <v>51100</v>
       </c>
     </row>
     <row r="343" ht="15.75" customHeight="1" s="4">
       <c r="C343" s="3" t="inlineStr">
         <is>
+          <t>ESPECIALIZACAO DESENVOLVIMENTO WEB</t>
+        </is>
+      </c>
+      <c r="E343" s="3" t="n">
+        <v>51200</v>
+      </c>
+    </row>
+    <row r="344" ht="15.75" customHeight="1" s="4">
+      <c r="C344" s="3" t="inlineStr">
+        <is>
           <t>ESPECIALIZACAO ENSINO DE MATEMATICA E FISICA</t>
         </is>
       </c>
-      <c r="E343" s="3" t="n">
+      <c r="E344" s="3" t="n">
         <v>51300</v>
       </c>
     </row>
-    <row r="344" ht="15.75" customHeight="1" s="4">
-      <c r="B344" s="3" t="inlineStr">
+    <row r="345" ht="15.75" customHeight="1" s="4">
+      <c r="B345" s="3" t="inlineStr">
         <is>
           <t>MESTRADO</t>
         </is>
-      </c>
-    </row>
-    <row r="345" ht="15.75" customHeight="1" s="4">
-      <c r="C345" s="3" t="inlineStr">
-        <is>
-          <t>MESTRADO</t>
-        </is>
-      </c>
-      <c r="E345" s="3" t="n">
-        <v>52000</v>
       </c>
     </row>
     <row r="346" ht="15.75" customHeight="1" s="4">
       <c r="C346" s="3" t="inlineStr">
         <is>
+          <t>MESTRADO</t>
+        </is>
+      </c>
+      <c r="E346" s="3" t="n">
+        <v>52000</v>
+      </c>
+    </row>
+    <row r="347" ht="15.75" customHeight="1" s="4">
+      <c r="C347" s="3" t="inlineStr">
+        <is>
           <t>MESTRADO PROFEPT</t>
         </is>
-      </c>
-    </row>
-    <row r="347" ht="15.75" customHeight="1" s="4">
-      <c r="D347" s="3" t="inlineStr">
-        <is>
-          <t>MESTRADO PROFEPT</t>
-        </is>
-      </c>
-      <c r="E347" s="3" t="n">
-        <v>52100</v>
       </c>
     </row>
     <row r="348" ht="15.75" customHeight="1" s="4">
       <c r="D348" s="3" t="inlineStr">
         <is>
-          <t>PROFEPT - SALA DA COORDENACAO</t>
+          <t>MESTRADO PROFEPT</t>
         </is>
       </c>
       <c r="E348" s="3" t="n">
-        <v>52101</v>
+        <v>52100</v>
       </c>
     </row>
     <row r="349" ht="15.75" customHeight="1" s="4">
       <c r="D349" s="3" t="inlineStr">
         <is>
+          <t>PROFEPT - SALA DA COORDENACAO</t>
+        </is>
+      </c>
+      <c r="E349" s="3" t="n">
+        <v>52101</v>
+      </c>
+    </row>
+    <row r="350" ht="15.75" customHeight="1" s="4">
+      <c r="D350" s="3" t="inlineStr">
+        <is>
           <t>PROFEPT - SALAS DE AULA</t>
         </is>
       </c>
-      <c r="E349" s="3" t="n">
+      <c r="E350" s="3" t="n">
         <v>52102</v>
-      </c>
-    </row>
-    <row r="350" ht="15.75" customHeight="1" s="4">
-      <c r="C350" s="3" t="inlineStr">
-        <is>
-          <t>MESTRADO PROFISSIONAL NUTRICAO E PRODUCAO ANIMAL</t>
-        </is>
-      </c>
-      <c r="E350" s="3" t="n">
-        <v>52200</v>
       </c>
     </row>
     <row r="351" ht="15.75" customHeight="1" s="4">
       <c r="C351" s="3" t="inlineStr">
         <is>
+          <t>MESTRADO PROFISSIONAL NUTRICAO E PRODUCAO ANIMAL</t>
+        </is>
+      </c>
+      <c r="E351" s="3" t="n">
+        <v>52200</v>
+      </c>
+    </row>
+    <row r="352" ht="15.75" customHeight="1" s="4">
+      <c r="C352" s="3" t="inlineStr">
+        <is>
           <t>MESTRADO PROFISSIONAL ALIMENTOS</t>
         </is>
       </c>
-      <c r="E351" s="3" t="n">
+      <c r="E352" s="3" t="n">
         <v>52300</v>
-      </c>
-    </row>
-    <row r="352" ht="15.75" customHeight="1" s="4">
-      <c r="B352" s="3" t="inlineStr">
-        <is>
-          <t>DOUTORADO</t>
-        </is>
-      </c>
-      <c r="E352" s="3" t="n">
-        <v>53000</v>
       </c>
     </row>
     <row r="353" ht="15.75" customHeight="1" s="4">
       <c r="B353" s="3" t="inlineStr">
         <is>
-          <t>NITTEC</t>
+          <t>DOUTORADO</t>
         </is>
       </c>
       <c r="E353" s="3" t="n">
-        <v>54000</v>
+        <v>53000</v>
       </c>
     </row>
     <row r="354" ht="15.75" customHeight="1" s="4">
       <c r="B354" s="3" t="inlineStr">
         <is>
-          <t>IF MAKER / NITTEC / IPCA</t>
+          <t>NITTEC</t>
         </is>
       </c>
       <c r="E354" s="3" t="n">
-        <v>54001</v>
+        <v>54000</v>
       </c>
     </row>
     <row r="355" ht="15.75" customHeight="1" s="4">
       <c r="B355" s="3" t="inlineStr">
         <is>
+          <t>IF MAKER / NITTEC / IPCA</t>
+        </is>
+      </c>
+      <c r="E355" s="3" t="n">
+        <v>54001</v>
+      </c>
+    </row>
+    <row r="356" ht="15.75" customHeight="1" s="4">
+      <c r="B356" s="3" t="inlineStr">
+        <is>
           <t>GERENCIA DE PESQUISA</t>
         </is>
       </c>
-      <c r="E355" s="3" t="n">
+      <c r="E356" s="3" t="n">
         <v>55000</v>
       </c>
     </row>
-    <row r="356" ht="15.75" customHeight="1" s="4">
-      <c r="A356" s="3" t="inlineStr">
+    <row r="357" ht="15.75" customHeight="1" s="4">
+      <c r="A357" s="3" t="inlineStr">
         <is>
           <t>DIRETORIA DE DESENVOLVIMENTO INSTITUCIONAL</t>
         </is>
-      </c>
-    </row>
-    <row r="357" ht="15.75" customHeight="1" s="4">
-      <c r="B357" s="3" t="inlineStr">
-        <is>
-          <t>DIRETORIA DE DESENVOLVIMENTO INSTITUCIONAL</t>
-        </is>
-      </c>
-      <c r="E357" s="3" t="n">
-        <v>60000</v>
       </c>
     </row>
     <row r="358" ht="15.75" customHeight="1" s="4">
       <c r="B358" s="3" t="inlineStr">
         <is>
+          <t>DIRETORIA DE DESENVOLVIMENTO INSTITUCIONAL</t>
+        </is>
+      </c>
+      <c r="E358" s="3" t="n">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="359" ht="15.75" customHeight="1" s="4">
+      <c r="B359" s="3" t="inlineStr">
+        <is>
           <t>PREFEITURA</t>
         </is>
-      </c>
-    </row>
-    <row r="359" ht="15.75" customHeight="1" s="4">
-      <c r="C359" s="3" t="inlineStr">
-        <is>
-          <t>PREFEITURA</t>
-        </is>
-      </c>
-      <c r="E359" s="3" t="n">
-        <v>61000</v>
       </c>
     </row>
     <row r="360" ht="15.75" customHeight="1" s="4">
       <c r="C360" s="3" t="inlineStr">
         <is>
-          <t>VIGILANCIA</t>
+          <t>PREFEITURA</t>
         </is>
       </c>
       <c r="E360" s="3" t="n">
-        <v>61100</v>
+        <v>61000</v>
       </c>
     </row>
     <row r="361" ht="15.75" customHeight="1" s="4">
       <c r="C361" s="3" t="inlineStr">
         <is>
-          <t>RECICLAGEM</t>
+          <t>VIGILANCIA</t>
         </is>
       </c>
       <c r="E361" s="3" t="n">
-        <v>61200</v>
+        <v>61100</v>
       </c>
     </row>
     <row r="362" ht="15.75" customHeight="1" s="4">
       <c r="C362" s="3" t="inlineStr">
         <is>
-          <t>SEÇÃO DE SERVICO DE APOIO</t>
+          <t>RECICLAGEM</t>
         </is>
       </c>
       <c r="E362" s="3" t="n">
-        <v>61300</v>
+        <v>61200</v>
       </c>
     </row>
     <row r="363" ht="15.75" customHeight="1" s="4">
       <c r="C363" s="3" t="inlineStr">
         <is>
-          <t>PREFEITURA - ESTACAO DE TRATAMENTO DE AGUA</t>
+          <t>SEÇÃO DE SERVICO DE APOIO</t>
         </is>
       </c>
       <c r="E363" s="3" t="n">
-        <v>61400</v>
+        <v>61300</v>
       </c>
     </row>
     <row r="364" ht="15.75" customHeight="1" s="4">
       <c r="C364" s="3" t="inlineStr">
         <is>
-          <t>PREFEITURA - MANUTEN. E DEPOS. MATER.CONSTRU</t>
+          <t>PREFEITURA - ESTACAO DE TRATAMENTO DE AGUA</t>
         </is>
       </c>
       <c r="E364" s="3" t="n">
-        <v>61401</v>
+        <v>61400</v>
       </c>
     </row>
     <row r="365" ht="15.75" customHeight="1" s="4">
       <c r="C365" s="3" t="inlineStr">
         <is>
-          <t>PREFEITURA - SERRALHERIA</t>
+          <t>PREFEITURA - MANUTEN. E DEPOS. MATER.CONSTRU</t>
         </is>
       </c>
       <c r="E365" s="3" t="n">
-        <v>61402</v>
+        <v>61401</v>
       </c>
     </row>
     <row r="366" ht="15.75" customHeight="1" s="4">
       <c r="C366" s="3" t="inlineStr">
         <is>
+          <t>PREFEITURA - SERRALHERIA</t>
+        </is>
+      </c>
+      <c r="E366" s="3" t="n">
+        <v>61402</v>
+      </c>
+    </row>
+    <row r="367" ht="15.75" customHeight="1" s="4">
+      <c r="C367" s="3" t="inlineStr">
+        <is>
           <t>PREFEITURA - CARPINTARIA</t>
         </is>
       </c>
-      <c r="E366" s="3" t="n">
+      <c r="E367" s="3" t="n">
         <v>61403</v>
       </c>
     </row>
-    <row r="367" ht="15.75" customHeight="1" s="4">
-      <c r="B367" s="3" t="inlineStr">
+    <row r="368" ht="15.75" customHeight="1" s="4">
+      <c r="B368" s="3" t="inlineStr">
         <is>
           <t>COORDENACAO GERAL DE PRODUCAO</t>
         </is>
-      </c>
-    </row>
-    <row r="368" ht="15.75" customHeight="1" s="4">
-      <c r="C368" s="3" t="inlineStr">
-        <is>
-          <t>COORDENACAO GERAL DE PRODUCAO</t>
-        </is>
-      </c>
-      <c r="E368" s="3" t="n">
-        <v>62000</v>
       </c>
     </row>
     <row r="369" ht="15.75" customHeight="1" s="4">
       <c r="C369" s="3" t="inlineStr">
         <is>
-          <t>MECANIZACAO AGRICOLA</t>
+          <t>COORDENACAO GERAL DE PRODUCAO</t>
         </is>
       </c>
       <c r="E369" s="3" t="n">
-        <v>62100</v>
+        <v>62000</v>
       </c>
     </row>
     <row r="370" ht="15.75" customHeight="1" s="4">
       <c r="C370" s="3" t="inlineStr">
         <is>
-          <t>POSTO DE VENDAS</t>
+          <t>MECANIZACAO AGRICOLA</t>
         </is>
       </c>
       <c r="E370" s="3" t="n">
-        <v>62200</v>
+        <v>62100</v>
       </c>
     </row>
     <row r="371" ht="15.75" customHeight="1" s="4">
       <c r="C371" s="3" t="inlineStr">
         <is>
-          <t>SECAO DE PROJETOS E PRODUCAO AGROINDUSTRIAL</t>
+          <t>POSTO DE VENDAS</t>
         </is>
       </c>
       <c r="E371" s="3" t="n">
-        <v>62300</v>
+        <v>62200</v>
       </c>
     </row>
     <row r="372" ht="15.75" customHeight="1" s="4">
       <c r="C372" s="3" t="inlineStr">
         <is>
-          <t>PADARIA</t>
+          <t>SECAO DE PROJETOS E PRODUCAO AGROINDUSTRIAL</t>
         </is>
       </c>
       <c r="E372" s="3" t="n">
-        <v>62301</v>
+        <v>62300</v>
       </c>
     </row>
     <row r="373" ht="15.75" customHeight="1" s="4">
       <c r="C373" s="3" t="inlineStr">
         <is>
-          <t>FRUTAS</t>
+          <t>PADARIA</t>
         </is>
       </c>
       <c r="E373" s="3" t="n">
-        <v>62302</v>
+        <v>62301</v>
       </c>
     </row>
     <row r="374" ht="15.75" customHeight="1" s="4">
       <c r="C374" s="3" t="inlineStr">
         <is>
-          <t>CARNES</t>
+          <t>FRUTAS</t>
         </is>
       </c>
       <c r="E374" s="3" t="n">
-        <v>62303</v>
+        <v>62302</v>
       </c>
     </row>
     <row r="375" ht="15.75" customHeight="1" s="4">
       <c r="C375" s="3" t="inlineStr">
         <is>
-          <t>INDUSTRIAS RURAIS</t>
+          <t>CARNES</t>
         </is>
       </c>
       <c r="E375" s="3" t="n">
-        <v>62304</v>
+        <v>62303</v>
       </c>
     </row>
     <row r="376" ht="15.75" customHeight="1" s="4">
       <c r="C376" s="3" t="inlineStr">
         <is>
-          <t>AGROINDUSTRIA - ESCRITORIO E ALMOXARIFADO</t>
+          <t>INDUSTRIAS RURAIS</t>
         </is>
       </c>
       <c r="E376" s="3" t="n">
-        <v>62305</v>
+        <v>62304</v>
       </c>
     </row>
     <row r="377" ht="15.75" customHeight="1" s="4">
       <c r="C377" s="3" t="inlineStr">
         <is>
-          <t>LATICINIO</t>
+          <t>AGROINDUSTRIA - ESCRITORIO E ALMOXARIFADO</t>
         </is>
       </c>
       <c r="E377" s="3" t="n">
-        <v>62306</v>
+        <v>62305</v>
       </c>
     </row>
     <row r="378" ht="15.75" customHeight="1" s="4">
       <c r="C378" s="3" t="inlineStr">
         <is>
+          <t>LATICINIO</t>
+        </is>
+      </c>
+      <c r="E378" s="3" t="n">
+        <v>62306</v>
+      </c>
+    </row>
+    <row r="379" ht="15.75" customHeight="1" s="4">
+      <c r="C379" s="3" t="inlineStr">
+        <is>
           <t>CALDEIRA</t>
         </is>
       </c>
-      <c r="E378" s="3" t="n">
+      <c r="E379" s="3" t="n">
         <v>62307</v>
       </c>
     </row>
-    <row r="379" ht="15.75" customHeight="1" s="4">
-      <c r="B379" s="3" t="inlineStr">
+    <row r="380" ht="15.75" customHeight="1" s="4">
+      <c r="B380" s="3" t="inlineStr">
         <is>
           <t>GERENCIA DE TECNOLOGIA DA INFORMACAO</t>
         </is>
-      </c>
-    </row>
-    <row r="380" ht="15.75" customHeight="1" s="4">
-      <c r="C380" s="3" t="inlineStr">
-        <is>
-          <t>GERENCIA DE TECNOLOGIA DA INFORMACAO</t>
-        </is>
-      </c>
-      <c r="E380" s="3" t="n">
-        <v>63000</v>
       </c>
     </row>
     <row r="381" ht="15.75" customHeight="1" s="4">
       <c r="C381" s="3" t="inlineStr">
         <is>
+          <t>GERENCIA DE TECNOLOGIA DA INFORMACAO</t>
+        </is>
+      </c>
+      <c r="E381" s="3" t="n">
+        <v>63000</v>
+      </c>
+    </row>
+    <row r="382" ht="15.75" customHeight="1" s="4">
+      <c r="C382" s="3" t="inlineStr">
+        <is>
           <t>TI - DATACENTER</t>
         </is>
       </c>
-      <c r="E381" s="3" t="n">
+      <c r="E382" s="3" t="n">
         <v>63001</v>
       </c>
     </row>
-    <row r="382" ht="15.75" customHeight="1" s="4">
-      <c r="A382" s="3" t="inlineStr">
+    <row r="383" ht="15.75" customHeight="1" s="4">
+      <c r="A383" s="3" t="inlineStr">
         <is>
           <t>DIRETOR GERAL</t>
         </is>
-      </c>
-    </row>
-    <row r="383" ht="15.75" customHeight="1" s="4">
-      <c r="B383" s="3" t="inlineStr">
-        <is>
-          <t>DIRETOR GERAL</t>
-        </is>
-      </c>
-      <c r="E383" s="3" t="n">
-        <v>70000</v>
       </c>
     </row>
     <row r="384" ht="15.75" customHeight="1" s="4">
       <c r="B384" s="3" t="inlineStr">
         <is>
-          <t>EMPRESTIMO DE BENS</t>
+          <t>DIRETOR GERAL</t>
         </is>
       </c>
       <c r="E384" s="3" t="n">
-        <v>70001</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="385" ht="15.75" customHeight="1" s="4">
       <c r="B385" s="3" t="inlineStr">
         <is>
-          <t>AUDITORIA INTERNA</t>
+          <t>EMPRESTIMO DE BENS</t>
         </is>
       </c>
       <c r="E385" s="3" t="n">
-        <v>70002</v>
+        <v>70001</v>
       </c>
     </row>
     <row r="386" ht="15.75" customHeight="1" s="4">
       <c r="B386" s="3" t="inlineStr">
         <is>
-          <t>ARQUIVO MORTO / GERAL</t>
+          <t>AUDITORIA INTERNA</t>
         </is>
       </c>
       <c r="E386" s="3" t="n">
-        <v>70003</v>
+        <v>70002</v>
       </c>
     </row>
     <row r="387" ht="15.75" customHeight="1" s="4">
       <c r="B387" s="3" t="inlineStr">
         <is>
-          <t>CESSAO DE BENS</t>
+          <t>ARQUIVO MORTO / GERAL</t>
         </is>
       </c>
       <c r="E387" s="3" t="n">
-        <v>70004</v>
+        <v>70003</v>
       </c>
     </row>
     <row r="388" ht="15.75" customHeight="1" s="4">
       <c r="B388" s="3" t="inlineStr">
         <is>
-          <t>SALAO NOBRE</t>
+          <t>CESSAO DE BENS</t>
         </is>
       </c>
       <c r="E388" s="3" t="n">
-        <v>70005</v>
+        <v>70004</v>
       </c>
     </row>
     <row r="389" ht="15.75" customHeight="1" s="4">
       <c r="B389" s="3" t="inlineStr">
         <is>
-          <t>GABINETE</t>
+          <t>SALAO NOBRE</t>
         </is>
       </c>
       <c r="E389" s="3" t="n">
-        <v>70006</v>
+        <v>70005</v>
       </c>
     </row>
     <row r="390" ht="15.75" customHeight="1" s="4">
       <c r="B390" s="3" t="inlineStr">
         <is>
+          <t>GABINETE</t>
+        </is>
+      </c>
+      <c r="E390" s="3" t="n">
+        <v>70006</v>
+      </c>
+    </row>
+    <row r="391" ht="15.75" customHeight="1" s="4">
+      <c r="B391" s="3" t="inlineStr">
+        <is>
           <t>GESTAO DE PESSOAS</t>
         </is>
       </c>
-      <c r="E390" s="3" t="n">
+      <c r="E391" s="3" t="n">
         <v>70007</v>
       </c>
     </row>
-    <row r="391" ht="15.75" customHeight="1" s="4">
-      <c r="B391" t="inlineStr">
+    <row r="392" ht="15.75" customHeight="1" s="4">
+      <c r="B392" s="0" t="inlineStr">
         <is>
           <t>CASA DOS INSTRUMENTOS MUSICAIS / CASA DO RAMON</t>
         </is>
       </c>
-      <c r="E391" t="n">
+      <c r="E392" s="0" t="n">
         <v>70008</v>
       </c>
     </row>
-    <row r="392" ht="15.75" customHeight="1" s="4">
-      <c r="B392" s="3" t="inlineStr">
+    <row r="393" ht="15.75" customHeight="1" s="4">
+      <c r="B393" s="3" t="inlineStr">
         <is>
           <t>FUNDACAO</t>
         </is>
-      </c>
-    </row>
-    <row r="393" ht="15.75" customHeight="1" s="4">
-      <c r="C393" s="3" t="inlineStr">
-        <is>
-          <t>FUNDACAO - REFEITORIO</t>
-        </is>
-      </c>
-      <c r="E393" s="3" t="n">
-        <v>70009</v>
       </c>
     </row>
     <row r="394" ht="15.75" customHeight="1" s="4">
       <c r="C394" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 1</t>
+          <t>FUNDACAO - REFEITORIO</t>
         </is>
       </c>
       <c r="E394" s="3" t="n">
-        <v>70011</v>
+        <v>70009</v>
       </c>
     </row>
     <row r="395" ht="15.75" customHeight="1" s="4">
       <c r="C395" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 2</t>
+          <t>FUNDACAO - DORMITORIO 1</t>
         </is>
       </c>
       <c r="E395" s="3" t="n">
-        <v>70012</v>
+        <v>70011</v>
       </c>
     </row>
     <row r="396" ht="15.75" customHeight="1" s="4">
       <c r="C396" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 3</t>
+          <t>FUNDACAO - DORMITORIO 2</t>
         </is>
       </c>
       <c r="E396" s="3" t="n">
-        <v>70013</v>
+        <v>70012</v>
       </c>
     </row>
     <row r="397" ht="15.75" customHeight="1" s="4">
       <c r="C397" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 4</t>
+          <t>FUNDACAO - DORMITORIO 3</t>
         </is>
       </c>
       <c r="E397" s="3" t="n">
-        <v>70014</v>
+        <v>70013</v>
       </c>
     </row>
     <row r="398" ht="15.75" customHeight="1" s="4">
       <c r="C398" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 5</t>
+          <t>FUNDACAO - DORMITORIO 4</t>
         </is>
       </c>
       <c r="E398" s="3" t="n">
-        <v>70015</v>
+        <v>70014</v>
       </c>
     </row>
     <row r="399" ht="15.75" customHeight="1" s="4">
       <c r="C399" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 6</t>
+          <t>FUNDACAO - DORMITORIO 5</t>
         </is>
       </c>
       <c r="E399" s="3" t="n">
-        <v>70016</v>
+        <v>70015</v>
       </c>
     </row>
     <row r="400" ht="15.75" customHeight="1" s="4">
       <c r="C400" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 7</t>
+          <t>FUNDACAO - DORMITORIO 6</t>
         </is>
       </c>
       <c r="E400" s="3" t="n">
-        <v>70017</v>
+        <v>70016</v>
       </c>
     </row>
     <row r="401" ht="15.75" customHeight="1" s="4">
       <c r="C401" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 8</t>
+          <t>FUNDACAO - DORMITORIO 7</t>
         </is>
       </c>
       <c r="E401" s="3" t="n">
-        <v>70018</v>
+        <v>70017</v>
       </c>
     </row>
     <row r="402" ht="15.75" customHeight="1" s="4">
       <c r="C402" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 9</t>
+          <t>FUNDACAO - DORMITORIO 8</t>
         </is>
       </c>
       <c r="E402" s="3" t="n">
-        <v>70019</v>
+        <v>70018</v>
       </c>
     </row>
     <row r="403" ht="15.75" customHeight="1" s="4">
       <c r="C403" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 10</t>
+          <t>FUNDACAO - DORMITORIO 9</t>
         </is>
       </c>
       <c r="E403" s="3" t="n">
-        <v>70020</v>
+        <v>70019</v>
       </c>
     </row>
     <row r="404" ht="15.75" customHeight="1" s="4">
       <c r="C404" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - DORMITORIO 11</t>
+          <t>FUNDACAO - DORMITORIO 10</t>
         </is>
       </c>
       <c r="E404" s="3" t="n">
-        <v>70021</v>
+        <v>70020</v>
       </c>
     </row>
     <row r="405" ht="15.75" customHeight="1" s="4">
       <c r="C405" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - HALL SEGUNDO ANDAR</t>
+          <t>FUNDACAO - DORMITORIO 11</t>
         </is>
       </c>
       <c r="E405" s="3" t="n">
-        <v>70022</v>
+        <v>70021</v>
       </c>
     </row>
     <row r="406" ht="15.75" customHeight="1" s="4">
       <c r="C406" s="3" t="inlineStr">
         <is>
-          <t>FUNDACAO - SALA SEGUNDO ANDAR</t>
+          <t>FUNDACAO - HALL SEGUNDO ANDAR</t>
         </is>
       </c>
       <c r="E406" s="3" t="n">
-        <v>70023</v>
+        <v>70022</v>
       </c>
     </row>
     <row r="407" ht="15.75" customHeight="1" s="4">
       <c r="C407" s="3" t="inlineStr">
         <is>
+          <t>FUNDACAO - SALA SEGUNDO ANDAR</t>
+        </is>
+      </c>
+      <c r="E407" s="3" t="n">
+        <v>70023</v>
+      </c>
+    </row>
+    <row r="408" ht="15.75" customHeight="1" s="4">
+      <c r="C408" s="3" t="inlineStr">
+        <is>
           <t>FUNDACAO - ANFITEATRO JARBAS FURTADO</t>
         </is>
       </c>
-      <c r="E407" s="3" t="n">
+      <c r="E408" s="3" t="n">
         <v>70010</v>
-      </c>
-    </row>
-    <row r="408" ht="15.75" customHeight="1" s="4">
-      <c r="B408" s="3" t="inlineStr">
-        <is>
-          <t>CENTRO DE VIVENCIA / CANTINA</t>
-        </is>
-      </c>
-      <c r="E408" s="3" t="n">
-        <v>70024</v>
       </c>
     </row>
     <row r="409" ht="15.75" customHeight="1" s="4">
       <c r="B409" s="3" t="inlineStr">
         <is>
+          <t>CENTRO DE VIVENCIA / CANTINA</t>
+        </is>
+      </c>
+      <c r="E409" s="3" t="n">
+        <v>70024</v>
+      </c>
+    </row>
+    <row r="410" ht="15.75" customHeight="1" s="4">
+      <c r="B410" s="3" t="inlineStr">
+        <is>
           <t>ALOJAMENTO - BLOCO C</t>
         </is>
-      </c>
-    </row>
-    <row r="410" ht="15.75" customHeight="1" s="4">
-      <c r="C410" s="3" t="inlineStr">
-        <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 1</t>
-        </is>
-      </c>
-      <c r="E410" s="3" t="n">
-        <v>70025</v>
       </c>
     </row>
     <row r="411" ht="15.75" customHeight="1" s="4">
       <c r="C411" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 2</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 1</t>
         </is>
       </c>
       <c r="E411" s="3" t="n">
-        <v>70026</v>
+        <v>70025</v>
       </c>
     </row>
     <row r="412" ht="15.75" customHeight="1" s="4">
       <c r="C412" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 3</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 2</t>
         </is>
       </c>
       <c r="E412" s="3" t="n">
-        <v>70027</v>
+        <v>70026</v>
       </c>
     </row>
     <row r="413" ht="15.75" customHeight="1" s="4">
       <c r="C413" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 4</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 3</t>
         </is>
       </c>
       <c r="E413" s="3" t="n">
-        <v>70028</v>
+        <v>70027</v>
       </c>
     </row>
     <row r="414" ht="15.75" customHeight="1" s="4">
       <c r="C414" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 5</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 4</t>
         </is>
       </c>
       <c r="E414" s="3" t="n">
-        <v>70029</v>
+        <v>70028</v>
       </c>
     </row>
     <row r="415" ht="15.75" customHeight="1" s="4">
       <c r="C415" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO C - QUARTO 6</t>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 5</t>
         </is>
       </c>
       <c r="E415" s="3" t="n">
-        <v>70030</v>
+        <v>70029</v>
       </c>
     </row>
     <row r="416" ht="15.75" customHeight="1" s="4">
       <c r="C416" s="3" t="inlineStr">
         <is>
+          <t>ALOJAMENTO - BLOCO C - QUARTO 6</t>
+        </is>
+      </c>
+      <c r="E416" s="3" t="n">
+        <v>70030</v>
+      </c>
+    </row>
+    <row r="417" ht="15.75" customHeight="1" s="4">
+      <c r="C417" s="3" t="inlineStr">
+        <is>
           <t>ALOJAMENTO - BLOCO C - QUARTO 7</t>
         </is>
       </c>
-      <c r="E416" s="3" t="n">
+      <c r="E417" s="3" t="n">
         <v>70031</v>
       </c>
     </row>
-    <row r="417" ht="15.75" customHeight="1" s="4">
-      <c r="B417" s="3" t="inlineStr">
+    <row r="418" ht="15.75" customHeight="1" s="4">
+      <c r="B418" s="3" t="inlineStr">
         <is>
           <t>ALOJAMENTO - BLOCO D</t>
         </is>
-      </c>
-    </row>
-    <row r="418" ht="15.75" customHeight="1" s="4">
-      <c r="C418" s="3" t="inlineStr">
-        <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 1</t>
-        </is>
-      </c>
-      <c r="E418" s="3" t="n">
-        <v>70032</v>
       </c>
     </row>
     <row r="419" ht="15.75" customHeight="1" s="4">
       <c r="C419" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 2</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 1</t>
         </is>
       </c>
       <c r="E419" s="3" t="n">
-        <v>70033</v>
+        <v>70032</v>
       </c>
     </row>
     <row r="420" ht="15.75" customHeight="1" s="4">
       <c r="C420" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 3</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 2</t>
         </is>
       </c>
       <c r="E420" s="3" t="n">
-        <v>70034</v>
+        <v>70033</v>
       </c>
     </row>
     <row r="421" ht="15.75" customHeight="1" s="4">
       <c r="C421" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 4</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 3</t>
         </is>
       </c>
       <c r="E421" s="3" t="n">
-        <v>70035</v>
+        <v>70034</v>
       </c>
     </row>
     <row r="422" ht="15.75" customHeight="1" s="4">
       <c r="C422" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 5</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 4</t>
         </is>
       </c>
       <c r="E422" s="3" t="n">
-        <v>70036</v>
+        <v>70035</v>
       </c>
     </row>
     <row r="423" ht="15.75" customHeight="1" s="4">
       <c r="C423" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 6</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 5</t>
         </is>
       </c>
       <c r="E423" s="3" t="n">
-        <v>70037</v>
+        <v>70036</v>
       </c>
     </row>
     <row r="424" ht="15.75" customHeight="1" s="4">
       <c r="C424" s="3" t="inlineStr">
         <is>
-          <t>ALOJAMENTO - BLOCO D - QUARTO 7</t>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 6</t>
         </is>
       </c>
       <c r="E424" s="3" t="n">
-        <v>70038</v>
+        <v>70037</v>
       </c>
     </row>
     <row r="425" ht="15.75" customHeight="1" s="4">
       <c r="C425" s="3" t="inlineStr">
         <is>
+          <t>ALOJAMENTO - BLOCO D - QUARTO 7</t>
+        </is>
+      </c>
+      <c r="E425" s="3" t="n">
+        <v>70038</v>
+      </c>
+    </row>
+    <row r="426" ht="15.75" customHeight="1" s="4">
+      <c r="C426" s="3" t="inlineStr">
+        <is>
           <t>ALOJAMENTO - GALPAO / DEPOSITO</t>
         </is>
       </c>
-      <c r="E425" s="3" t="n">
+      <c r="E426" s="3" t="n">
         <v>70039</v>
-      </c>
-    </row>
-    <row r="426" ht="15.75" customHeight="1" s="4">
-      <c r="B426" s="0" t="inlineStr">
-        <is>
-          <t>SALA WEB RADIO (ALOJAMENTO / BLOCO B / SALA 1)</t>
-        </is>
-      </c>
-      <c r="E426" s="0" t="n">
-        <v>70040</v>
       </c>
     </row>
     <row r="427" ht="15.75" customHeight="1" s="4">
       <c r="B427" s="0" t="inlineStr">
         <is>
+          <t>SALA WEB RADIO (ALOJAMENTO / BLOCO B / SALA 1)</t>
+        </is>
+      </c>
+      <c r="E427" s="0" t="n">
+        <v>70040</v>
+      </c>
+    </row>
+    <row r="428" ht="15.75" customHeight="1" s="4">
+      <c r="B428" s="0" t="inlineStr">
+        <is>
           <t>CAPELA / IGREJINHA</t>
         </is>
       </c>
-      <c r="E427" s="0" t="n">
+      <c r="E428" s="0" t="n">
         <v>70041</v>
       </c>
     </row>
-    <row r="428" ht="15.75" customHeight="1" s="4">
-      <c r="B428" s="3" t="inlineStr">
+    <row r="429" ht="15.75" customHeight="1" s="4">
+      <c r="B429" s="3" t="inlineStr">
         <is>
           <t>COMUNICACAO</t>
         </is>
-      </c>
-    </row>
-    <row r="429" ht="15.75" customHeight="1" s="4">
-      <c r="C429" s="3" t="inlineStr">
-        <is>
-          <t>COMUNICACAO</t>
-        </is>
-      </c>
-      <c r="E429" s="3" t="n">
-        <v>71000</v>
       </c>
     </row>
     <row r="430" ht="15.75" customHeight="1" s="4">
       <c r="C430" s="3" t="inlineStr">
         <is>
-          <t>SALA DA COMUNICACAO - FUNDACAO</t>
+          <t>COMUNICACAO</t>
         </is>
       </c>
       <c r="E430" s="3" t="n">
-        <v>71002</v>
+        <v>71000</v>
       </c>
     </row>
     <row r="431" ht="15.75" customHeight="1" s="4">
       <c r="C431" s="3" t="inlineStr">
         <is>
+          <t>SALA DA COMUNICACAO - FUNDACAO</t>
+        </is>
+      </c>
+      <c r="E431" s="3" t="n">
+        <v>71002</v>
+      </c>
+    </row>
+    <row r="432" ht="15.75" customHeight="1" s="4">
+      <c r="C432" s="3" t="inlineStr">
+        <is>
           <t>SALA DA COMUNICACAO - PREDIO ADMINISTRATIVO</t>
         </is>
       </c>
-      <c r="E431" s="3" t="n">
+      <c r="E432" s="3" t="n">
         <v>71001</v>
       </c>
     </row>
-    <row r="432" ht="15.75" customHeight="1" s="4"/>
     <row r="433" ht="15.75" customHeight="1" s="4"/>
     <row r="434" ht="15.75" customHeight="1" s="4"/>
     <row r="435" ht="15.75" customHeight="1" s="4"/>

</xml_diff>